<commit_message>
docs(qa): update QC result sheet after bug fixes and re-verification
Complete 840-point run plus re-test of the fixed items: Lulus 572, Gagal 25, Sebagian 199, Tidak Dapat Diuji 44. Changed rows keep the previous result in their note.
</commit_message>
<xml_diff>
--- a/Required Document/QC_Claude_Hasil.xlsx
+++ b/Required Document/QC_Claude_Hasil.xlsx
@@ -40,7 +40,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -64,11 +64,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
@@ -85,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -95,7 +90,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -519,13 +513,13 @@
         <v>179</v>
       </c>
       <c r="C2" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -534,7 +528,7 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -547,13 +541,13 @@
         <v>135</v>
       </c>
       <c r="C3" t="n">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F3" t="n">
         <v>4</v>
@@ -562,7 +556,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -575,13 +569,13 @@
         <v>51</v>
       </c>
       <c r="C4" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D4" t="n">
         <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -590,7 +584,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -603,22 +597,22 @@
         <v>100</v>
       </c>
       <c r="C5" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="D5" t="n">
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -631,22 +625,22 @@
         <v>61</v>
       </c>
       <c r="C6" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -659,13 +653,13 @@
         <v>55</v>
       </c>
       <c r="C7" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -674,7 +668,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -687,13 +681,13 @@
         <v>49</v>
       </c>
       <c r="C8" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -715,7 +709,7 @@
         <v>38</v>
       </c>
       <c r="C9" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
@@ -724,7 +718,7 @@
         <v>10</v>
       </c>
       <c r="F9" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -743,10 +737,10 @@
         <v>64</v>
       </c>
       <c r="C10" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
         <v>9</v>
@@ -799,10 +793,10 @@
         <v>40</v>
       </c>
       <c r="C12" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
         <v>3</v>
@@ -879,7 +873,7 @@
           <t>Guest membuka beranda → katalog → detail produk; pilih warna/ukuran, upload desain sendiri, Tambah ke Keranjang → diminta login</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -929,7 +923,7 @@
           <t>Login → keranjang berisi item yang tadi ditambahkan (tidak hilang)</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -1679,7 +1673,7 @@
           <t>Refund dilakukan manual &amp; dikomunikasikan lewat chat (BR-006/015) — alur manual terdokumentasi</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -1754,7 +1748,7 @@
           <t>Komplain kualitas lewat Chat dalam 7 hari setelah Selesai ditangani manual (BR-016); setelah 7 hari dianggap final</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -1779,7 +1773,7 @@
           <t>Produksi ulang gratis jika salah produksi (BR-011) — alur manual terdokumentasi</t>
         </is>
       </c>
-      <c r="D38" s="7" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -1829,14 +1823,14 @@
           <t>Blokir hak cipta: akun tidak bisa login sama sekali; komisi terhutang berubah "Ditahan"</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Blokir hak cipta: komisi berubah ditahan (diverifikasi), TETAPI akun masih bisa login (200) -&gt; AuthService::attemptLogin tidak memeriksa users.status (Banned/Nonaktif).</t>
+          <t>banned: Verifikasi ulang setelah perbaikan: akun banned ditolak saat login (HTTP 422) dan sesi lama ditolak (HTTP 403); komisi ditahan tetap sesuai uji sebelumnya | Sebelumnya (Gagal): Blokir hak cipta: komisi berubah ditahan (diverifikasi), TETAPI akun masih bisa login (200) -&gt; AuthService::at</t>
         </is>
       </c>
     </row>
@@ -1879,14 +1873,14 @@
           <t>Item wishlist/keranjang dari desain creator terblokir ditandai tidak tersedia &amp; tidak bisa di-checkout (BR-024)</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>BR-024: setelah creator diblokir, item keranjang desainnya tetap is_available=true dan checkout berhasil (201); CartItemResource::is_available hanya melihat product.is_active, tidak status desain/creator.</t>
+          <t>BR-024 desain creator diblokir: Verifikasi ulang setelah perbaikan: item desain creator #11: is_available true -&gt; false setelah creator di-ban; POST /checkout -&gt; HTTP 422 (ditolak). Dipulihkan. | Sebelumnya (Gagal): BR-024: setelah creator diblokir, item keranjang desainnya tetap is_available=true dan checkout berhasil (201)</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2298,7 @@
           <t>Dua browser (customer &amp; admin): pesan customer muncul di admin tanpa refresh dan sebaliknya</t>
         </is>
       </c>
-      <c r="D59" s="7" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -2329,7 +2323,7 @@
           <t>Aksi admin (setujui desain/ubah status) memunculkan notifikasi di browser customer/creator tanpa refresh</t>
         </is>
       </c>
-      <c r="D60" s="7" t="inlineStr">
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -2354,7 +2348,7 @@
           <t>Putus-sambung internet: koneksi realtime tersambung ulang &amp; tidak ada pesan hilang/ganda</t>
         </is>
       </c>
-      <c r="D61" s="7" t="inlineStr">
+      <c r="D61" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -2429,7 +2423,7 @@
           <t>Ganti bahasa di tengah checkout → data keranjang &amp; alamat tidak hilang</t>
         </is>
       </c>
-      <c r="D64" s="7" t="inlineStr">
+      <c r="D64" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -2552,7 +2546,7 @@
           <t>Scheduler benar-benar berjalan di server produksi (cron `* * * * * schedule:run` atau service) — tanpa ini ketiga job tidak jalan</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -2927,7 +2921,7 @@
           <t>URL notifikasi terdaftar di dashboard Midtrans mengarah ke domain backend yang benar (api.harmoniclothing.com)</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -3277,7 +3271,7 @@
           <t>Locale: header Accept-Language dan ?lang diterapkan ke nama produk/kategori &amp; pesan</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -3402,7 +3396,7 @@
           <t>Email verifikasi: pengirim hello@harmoniclothing.com, subjek benar, tombol "Verifikasi Email", tautan ke frontend /verify-email berisi id/hash/expires/signature yang valid</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -3452,7 +3446,7 @@
           <t>Isi email mengikuti locale (ID/EN); tampilan rapi di Gmail/Outlook/mobile</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -3477,7 +3471,7 @@
           <t>Email tidak masuk spam pada kotak masuk uji (SPF/DKIM/DMARC lulus untuk domain pengirim)</t>
         </is>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -3502,7 +3496,7 @@
           <t>Email terkirim ke alamat mana pun (bukan hanya pemilik akun Resend) — domain terverifikasi</t>
         </is>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -3527,7 +3521,7 @@
           <t>Kegagalan Resend tidak membuat registrasi/lupa password crash 500 (ditangani/dicatat)</t>
         </is>
       </c>
-      <c r="D42" s="7" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -3602,7 +3596,7 @@
           <t>Kanal notifikasi privat per user; user lain tidak dapat subscribe</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -3627,7 +3621,7 @@
           <t>Otorisasi /broadcasting/auth memakai cookie sesi + CSRF dan lewat domain yang sama</t>
         </is>
       </c>
-      <c r="D46" s="7" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -3802,7 +3796,7 @@
           <t>Berkas yang dihapus/diganti tidak meninggalkan referensi rusak</t>
         </is>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -3952,7 +3946,7 @@
           <t>Migrasi database terkini sudah dijalankan; tidak ada migrasi tertunda</t>
         </is>
       </c>
-      <c r="D59" s="7" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -4177,7 +4171,7 @@
           <t>`pnpm build` sukses (semua rute terdaftar)</t>
         </is>
       </c>
-      <c r="D68" s="7" t="inlineStr">
+      <c r="D68" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -4450,14 +4444,14 @@
           <t>Akun banned/nonaktif tidak dapat login &amp; sesi aktif ditolak</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>TEMUAN KRITIS: user dengan status 'banned' (ban + copyright_violation) tetap bisa login baru (200) dan sesi lamanya tetap valid (/me 200). UserStatus Banned/Nonaktif hanya ditulis di CreatorService::ban, tidak pernah dicek di login/middleware. Ban biasa memang hanya mencabut akses /creator/* (403, sesuai desain). Perlu cek login &amp; middleware auth.</t>
+          <t>banned login &amp; sesi: Verifikasi ulang setelah perbaikan: login user banned HTTP 422 (ditolak); sesi aktif lalu user di-ban: /me 200 -&gt; 403; login ulang 422. Dipulihkan. | Sebelumnya (Gagal): TEMUAN KRITIS: user dengan status 'banned' (ban + copyright_violation) tetap bisa login baru (200) dan sesi la</t>
         </is>
       </c>
     </row>
@@ -4925,7 +4919,7 @@
           <t>Mixed content: semua aset dimuat lewat HTTPS</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -5225,7 +5219,7 @@
           <t>Hak penghapusan/koreksi data dapat diajukan lewat kontak (sesuai kebijakan privasi)</t>
         </is>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -5598,14 +5592,14 @@
           <t>Jika data produk/desain kosong atau API gagal, section menampilkan empty/error state (bukan crash)</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Browser QC (localhost:3001 + backend QC): backend dimatikan: /catalog tetap menampilkan skeleton &gt;10 detik tanpa pesan error/tombol Coba Lagi (17 request ERR_CONNECTION_REFUSED).</t>
+          <t>backend mati: /catalog: Verifikasi ulang setelah perbaikan: backend mati: /catalog menampilkan 'Terjadi kesalahan' + tombol Coba Lagi (bukan skeleton selamanya) | Sebelumnya (Gagal): Browser QC (localhost:3001 + backend QC): backend dimatikan: /catalog tetap menampilkan skeleton &gt;10 detik tan</t>
         </is>
       </c>
     </row>
@@ -5698,14 +5692,14 @@
           <t>Tampilan rapi di mobile (375px), tablet (768px), dan desktop (1280px+)</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): overflow tablet 768: scroll horizontal pada 768px: beranda=38px, katalog=42px, marketplace=42px, about=38px (beranda: elemen hero 'hidden animate-fade-slide-in md:' melebar sampai x=806) | Bukti lain: UI (Playwright, Edge headless, :3001 + backend QC): responsif beranda: overflow: 375:0, 768:38, 1280:0, 1920:0 | Bukti lain: Browser QC (loc</t>
+          <t>Verifikasi ulang setelah perbaikan: 768x1024 dan 800x375 tanpa scroll horizontal pada /, /catalog, /marketplace (tab Desain &amp; Kreator), /about, /faq, detail produk, detail desain. Perbaikan: header desktop pindah ke breakpoint lg (menu hamburger di bawah 1024px), toolbar daftar dan kolom detail produk/desain bertumpuk sampai lg. | Sebelumnya (Gagal): overflow tablet 768: Verifikasi ulang setelah perbaikan: /=0, /catalog=0, /marketplace=0, /about=0, /faq=0, /c</t>
         </is>
       </c>
     </row>
@@ -6373,14 +6367,14 @@
           <t>Loading skeleton tampil saat data dimuat; error state + tombol "Coba Lagi" tampil saat API gagal</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): error state API gagal (marketplace/katalog): skeleton tampil (Error #41); error state + 'Coba Lagi' TIDAK tampil saat API gagal (Error #11, #22)</t>
+          <t>error state API gagal: Verifikasi ulang setelah perbaikan: marketplace dengan API 500: error state + Coba Lagi tampil | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): error state API gagal (marketplace/katalog): skeleton tamp</t>
         </is>
       </c>
     </row>
@@ -6473,12 +6467,16 @@
           <t>Hasil kosong menampilkan pesan "Belum ada kreator ditemukan" + reset</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr"/>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>tab kreator kosong: Verifikasi ulang setelah perbaikan: tab Kreator kosong menampilkan 'Belum ada kreator ditemukan.' (tombol reset hanya tampil bila ada pencarian/filter aktif) | Sebelumnya (Gagal): Browser QC (Playwright, putaran 2): tab Kreator dengan hasil kosong hanya menampilkan 'Menampilkan 0 dari 0 kr</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -6494,12 +6492,16 @@
           <t>Foto profil kreator tampil (bukan broken image); kreator tanpa foto menampilkan avatar default</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Browser QC (Playwright, putaran 2): tab Kreator memuat 7 kartu kreator; seluruh 7 kreator seed tidak punya foto (photo_url null) dan kartu tampil tanpa elemen &lt;img&gt; rusak (avatar default). Kasus kreator dengan foto nyata tidak ada di data seed sehingga belum diuji.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -6590,12 +6592,16 @@
           <t>Tombol "Lihat Portofolio" membuka link portofolio (tab baru) &amp; hanya tampil bila diisi</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): tombol Lihat Portofolio: tidak ada kreator dengan portfolio_url di data seed; dengan portofolio: tidak ada data; tanpa portofolio: tombol=0</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -6611,12 +6617,16 @@
           <t>Statistik (Desain, Rating, Total Terjual) sesuai data nyata</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr"/>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): statistik profil creator: UI: Desain / Rating / Total Terjual / Desain oleh Balistreri-Abernathy (3); kunci API: name,photo_url,bio,portfolio_url,slug,since,designs; kecocokan angka dengan database belum dihitung ulang</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -6657,12 +6667,16 @@
           <t>Kreator tanpa desain menampilkan "Belum ada desain yang dipublikasikan"</t>
         </is>
       </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr"/>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): kreator tanpa desain: daftar desain kosong -&gt; 'Belum ada desain yang dipublikasikan.'</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -6828,12 +6842,16 @@
           <t>Opsi filter (warna/ukuran/material) berasal dari data nyata katalog; "Semua" &amp; "Reset" berfungsi</t>
         </is>
       </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr"/>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>opsi filter warna: Verifikasi ulang setelah perbaikan: filter Warna berupa swatch dengan nama aksesibel: Hitam, Merah QC, Navy, Putih; filter Ukuran=5 opsi; (koreksi: sebelumnya salah dilaporkan 'kosong', yang kurang hanya aria-label) | Sebelumnya (Sebagian): Browser QC (Playwright, putaran 2): filter /catalog: Ukuran (L, M, S, XL, XXL) dan Material (Cotton Combed 24s</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -6949,12 +6967,16 @@
           <t>Filter via URL dari footer (mis. kategori T-Shirt) menghasilkan hasil benar</t>
         </is>
       </c>
-      <c r="D68" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr"/>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Browser QC (Playwright, putaran 2): tautan footer 'T-Shirt' -&gt; /catalog?kategori=t-shirt menghasilkan 'Menampilkan 0 dari 10 produk': slug kategori di footer tidak cocok dengan kategori data QC (seed faker: Dolorum ipsam, dst.), jadi hasil filter benar hanya bisa dipastikan dengan kategori produksi 'T-Shirt'.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -7045,14 +7067,14 @@
           <t>Loading skeleton &amp; error state + "Coba Lagi" tampil sesuai kondisi</t>
         </is>
       </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): skeleton &amp; error state katalog: skeleton tampil; error state + 'Coba Lagi' tidak tampil saat API gagal (Error #11)</t>
+          <t>skeleton &amp; error state katalog: Verifikasi ulang setelah perbaikan: skeleton saat loading (9 elemen) dan error state saat API 500 | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): skeleton &amp; error state katalog: skeleton tampil; error sta</t>
         </is>
       </c>
     </row>
@@ -7095,12 +7117,16 @@
           <t>Galeri gambar berganti sesuai warna yang dipilih; thumbnail dapat diklik</t>
         </is>
       </c>
-      <c r="D74" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr"/>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): galeri berganti sesuai warna: warna tersedia=; gambar utama berubah saat ganti warna=false; jumlah gambar=9; mockup seed memakai placeholder sama sehingga perubahan visual tidak dapat dibuktikan penuh</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -7191,12 +7217,16 @@
           <t>Area upload "Upload Desain Sendiri (opsional)": file PNG/JPG ≤ 20MB berhasil, status berubah "File terunggah", dapat diganti</t>
         </is>
       </c>
-      <c r="D78" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr"/>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): upload desain sendiri di detail produk: PNG 300x300 diunggah -&gt; 'File terunggah — klik untuk ganti'</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -7212,12 +7242,16 @@
           <t>Upload file salah format/terlalu besar menampilkan pesan error "Gagal mengunggah file"</t>
         </is>
       </c>
-      <c r="D79" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr"/>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): upload salah format ditolak: tidak ada pesan error terdeteksi untuk berkas .txt: Upload Desain Sendiri (opsional) / Klik atau drag file di sini (PNG/SVG, maks 20MB)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -7483,12 +7517,16 @@
           <t>Tab Ulasan: daftar ulasan (nama pembeli, bintang, komentar, tanggal) + paginasi; kosong → "Belum ada ulasan"</t>
         </is>
       </c>
-      <c r="D90" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr"/>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): tab ulasan: API ulasan=5; UI: 3.4 (5 ulasan) / Ulasan (5); kosong -&gt; 'tidak terdeteksi'</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -7654,12 +7692,16 @@
           <t>Preview menampilkan desain di atas produk yang dipilih (bukan gambar rusak)</t>
         </is>
       </c>
-      <c r="D97" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E97" s="2" t="inlineStr"/>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): preview desain di atas produk: 10 gambar di detail desain termuat semua (tidak ada gambar rusak)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -7775,12 +7817,16 @@
           <t>Desain tanpa produk yang cocok menampilkan "Belum ada produk yang tersedia untuk desain ini"</t>
         </is>
       </c>
-      <c r="D102" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E102" s="2" t="inlineStr"/>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): desain tanpa produk cocok: pesan 'Belum ada produk yang tersedia untuk desain ini' tidak terdeteksi: Pilih Produk / Pilih Warna Produk: Hitam</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -7821,12 +7867,16 @@
           <t>"Koleksi Lainnya" menampilkan desain lain milik creator; "Lihat Semua →" berfungsi</t>
         </is>
       </c>
-      <c r="D104" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr"/>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): Koleksi Lainnya: bagian 'Koleksi Lainnya' tampil; 'Lihat Semua' berfungsi: /marketplace?kategori=placeat-saepe -&gt; /marketplace</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -7917,12 +7967,16 @@
           <t>Ikon wishlist desain berfungsi</t>
         </is>
       </c>
-      <c r="D108" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E108" s="2" t="inlineStr"/>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): ikon wishlist desain: wishlist 1 -&gt; 2 -&gt; 1 (toggle on/off tersimpan di server)</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -7963,12 +8017,16 @@
           <t>Section "Untuk Kreator Lokal" &amp; tombol "Jadi Kreator" berfungsi (guest → login/registrasi, user → /account/become-creator)</t>
         </is>
       </c>
-      <c r="D110" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="inlineStr"/>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>Browser QC (Playwright, putaran 2): bagian 'Untuk Kreator Lokal' tampil; tombol 'Jadi Kreator': guest -&gt; modal login/registrasi, user login -&gt; /account/become-creator.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -8509,12 +8567,16 @@
           <t>Tautan dari checkbox registrasi membuka halaman ini (tab baru) tanpa menutup form</t>
         </is>
       </c>
-      <c r="D132" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E132" s="2" t="inlineStr"/>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): tautan privacy dari registrasi: tautan /legal/privacy-policy target=_blank; form registrasi tetap terbuka=true; tab baru=false</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -8580,12 +8642,16 @@
           <t>Tautan dari checkbox registrasi &amp; pengajuan creator membuka halaman ini</t>
         </is>
       </c>
-      <c r="D135" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E135" s="2" t="inlineStr"/>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>Browser QC (Playwright, putaran 2): checkbox registrasi memiliki tautan /legal/terms; tetapi checkbox 'Saya menyetujui Syarat &amp; Ketentuan Creator' di /account/become-creator berupa teks biasa tanpa tautan ke halaman Syarat &amp; Ketentuan.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -8701,14 +8767,14 @@
           <t>Login akun yang di-ban/nonaktif ditolak dengan pesan yang sesuai</t>
         </is>
       </c>
-      <c r="D140" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): login akun banned: akun banned berhasil login lewat UI | Bukti lain: Akun banned (copyright) tetap bisa login dan memakai sesi (sheet Keamanan #8) -&gt; penolakan login akun banned tidak berfungsi.</t>
+          <t>login akun banned via UI: Verifikasi ulang setelah perbaikan: login akun banned lewat UI ditolak dengan pesan 'Akun Anda telah diblokir. Hubungi admin Harmoni Clothing untuk informasi lebih lanjut.'; modal tetap terbuka=true | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): login akun banned: akun banned berhasil login lewat UI | B</t>
         </is>
       </c>
     </row>
@@ -10530,14 +10596,14 @@
           <t>Tombol "Pindahkan ke wishlist" memindahkan item &amp; menampilkan toast</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): pindahkan ke wishlist: wishlist 0, keranjang 1 | Bukti lain: UI (Playwright, Edge headless, :3001 + backend QC): pindahkan ke wishlist: wishlist 4-&gt;4, keranjang 2</t>
+          <t>pindahkan ke wishlist: Verifikasi ulang setelah perbaikan: keranjang 3 -&gt; 2, wishlist 1 -&gt; 2 (produk dipindah, toast sukses) | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): pindahkan ke wishlist: wishlist 0, keranjang 1 | Bukti lai</t>
         </is>
       </c>
     </row>
@@ -10630,12 +10696,16 @@
           <t>Tidak ada infinite re-render / lag saat memilih item (regresi bug lama)</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr"/>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): cart: tanpa re-render tak terbatas saat memilih item: 4 checkbox; 8 klik berurutan selesai 1659 ms; error 'Maximum update depth'=0; console error total=2</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -10951,7 +11021,7 @@
           <t>Pembayaran Midtrans (Sandbox): kartu, VA bank, e-wallet/QRIS tersedia &amp; dapat dibayar</t>
         </is>
       </c>
-      <c r="D49" s="7" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -11001,7 +11071,7 @@
           <t>Menutup halaman pembayaran tanpa bayar → pesanan tetap "Belum Dibayar" &amp; bisa dibayar ulang dari detail pesanan (jika tersedia)</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -11276,12 +11346,16 @@
           <t>Upload desain sendiri (opsional) berfungsi; link pilih desain marketplace berfungsi; catatan opsional tersimpan</t>
         </is>
       </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr"/>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): bulk order: upload desain, pilih marketplace, catatan: halaman bulk order: input upload desain=1, tautan pilih desain marketplace=1, kolom catatan=1; penyimpanan catatan sampai ke pesanan tidak diverifikasi (butuh checkout bulk + Midtrans)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -11622,12 +11696,16 @@
           <t>Paginasi/muat lebih banyak berfungsi bila pesanan banyak</t>
         </is>
       </c>
-      <c r="D76" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr"/>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): paginasi riwayat pesanan: UI menampilkan 20 dari 21 pesanan; kontrol paginasi=1</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -11793,14 +11871,14 @@
           <t>Pesanan "Belum Dibayar": tautan/tombol bayar (jika ada) berfungsi; setelah 24 jam otomatis Dibatalkan (BR-017)</t>
         </is>
       </c>
-      <c r="D83" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): pesanan belum dibayar: bayar ulang: detail pesanan 'Belum Dibayar' tidak memiliki tombol/tautan bayar atau batal; pelanggan tidak dapat membayar ulang dari UI</t>
+          <t xml:space="preserve">Verifikasi ulang setelah perbaikan: detail pesanan HC-20261013-0469 (Belum Dibayar): tombol 'Bayar Sekarang' dan 'Batalkan Pesanan' tampil; tanpa tautan Snap -&gt; pesan 'Tautan pembayaran belum tersedia...'; dengan tautan tersimpan -&gt; diarahkan ke URL Snap (POST /orders/{id}/pay); Batalkan -&gt; status dibatalkan. Pesanan dipulihkan. Tombol 'Lihat Invoice' kini disembunyikan untuk pesanan Belum Dibayar. | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): pesanan belum dibayar: bayar ulang: detail pesanan 'Belum </t>
         </is>
       </c>
     </row>
@@ -11918,14 +11996,14 @@
           <t>Tautan "Lihat Invoice" membuka invoice pesanan</t>
         </is>
       </c>
-      <c r="D88" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UI (Playwright, Edge headless, :3001 + backend QC): Lihat Invoice: halaman invoice menampilkan 'Terjadi kesalahan' (crash: order.items tidak ada di respons invoice) | Bukti lain: Browser QC (login test@example.com): halaman invoice /account/orders/{id}/invoice menampilkan error boundary 'Terjadi kesalahan' karena API </t>
+          <t>Lihat Invoice: Verifikasi ulang setelah perbaikan: halaman invoice termuat tanpa crash: no. INV-20261013-1363, baris item, subtotal/ongkir/total; page error=0; tombol Cetak ada=true | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): Lihat Invoice: halaman invoice menampilkan 'Terjadi kesala</t>
         </is>
       </c>
     </row>
@@ -11943,12 +12021,16 @@
           <t>Pratinjau desain per item (file yang dikirim customer / desain marketplace) tampil benar</t>
         </is>
       </c>
-      <c r="D89" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="inlineStr"/>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>Browser QC (Playwright, putaran 2): detail pesanan HC-20261013-7551 (item dengan desain marketplace): pratinjau desain tampil sebagai thumbnail kecil 64px (placeholder seed 'designs/thumbnails/placeholder.png'); API mengirim design_file_url dan custom_design_url. File desain unggahan customer sendiri belum diuji.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -12014,14 +12096,14 @@
           <t>Nomor invoice, tanggal terbit, data penjual &amp; pembeli, rincian item, subtotal, ongkir, total dibayar sesuai pesanan</t>
         </is>
       </c>
-      <c r="D92" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Browser QC (login test@example.com): invoice tidak dapat dirender (lihat #87): API /orders/{id}/invoice memuat invoice_number &amp; order tanpa items/alamat/pembeli.</t>
+          <t>Invoice dirender: Verifikasi ulang setelah perbaikan: API /orders/{id}/invoice kini memuat order.items (nama produk, qty, subtotal) sehingga halaman invoice dapat dirender; lihat #87 | Sebelumnya (Gagal): Browser QC (login test@example.com): invoice tidak dapat dirender (lihat #87): API /orders/{id}/invoice memuat</t>
         </is>
       </c>
     </row>
@@ -12039,14 +12121,14 @@
           <t>Badge "Lunas" hanya untuk pesanan yang sudah dibayar</t>
         </is>
       </c>
-      <c r="D93" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): badge Lunas: halaman invoice tidak dapat dirender (crash, Customer #87) sehingga badge 'Lunas' tidak dapat diverifikasi</t>
+          <t xml:space="preserve">Badge Lunas: Verifikasi ulang setelah perbaikan: badge 'Lunas' tampil di halaman invoice | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): badge Lunas: halaman invoice tidak dapat dirender (crash, </t>
         </is>
       </c>
     </row>
@@ -12089,14 +12171,14 @@
           <t>Tombol Print membuka dialog cetak dengan tata letak rapi; tombol Kembali berfungsi</t>
         </is>
       </c>
-      <c r="D95" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): Print invoice: halaman invoice crash (Customer #87) -&gt; tombol Print/Kembali tidak dapat diuji</t>
+          <t>Verifikasi ulang setelah perbaikan: halaman invoice termuat; tombol 'Print' ada dan memanggil window.print() (dialog cetak browser tidak diotomasi). | Sebelumnya (Gagal): Print invoice: Verifikasi ulang setelah perbaikan: tombol cetak tidak ditemukan | Sebelumnya (Sebagian): UI (P</t>
         </is>
       </c>
     </row>
@@ -12264,12 +12346,16 @@
           <t>Batal pada dialog crop tidak mengubah foto lama</t>
         </is>
       </c>
-      <c r="D102" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E102" s="2" t="inlineStr"/>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): batal crop foto tidak mengubah foto lama: dialog crop (Simpan Foto) dibatalkan; src foto profil tetap sama</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -12310,12 +12396,16 @@
           <t>Foto profil tidak broken (URL R2/storage benar) setelah reload</t>
         </is>
       </c>
-      <c r="D104" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr"/>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): foto profil tidak broken setelah reload: user tidak punya foto (kunci /me: id,name,email,phone,photo_url,role,status,email_verified_at); unggah foto nyata tidak diuji</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -13031,7 +13121,7 @@
           <t>Balasan admin muncul real-time di panel; badge/indikator pesan baru bekerja</t>
         </is>
       </c>
-      <c r="D133" s="7" t="inlineStr">
+      <c r="D133" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -13106,7 +13196,7 @@
           <t>Tidak ada pesan ganda saat koneksi realtime putus-sambung</t>
         </is>
       </c>
-      <c r="D136" s="7" t="inlineStr">
+      <c r="D136" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -13329,12 +13419,16 @@
           <t>Pindah antara area Customer ↔ Creator tanpa logout; sesi tetap</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): pindah Customer &lt;-&gt; Creator tanpa logout: /account/profile -&gt; /creator/dashboard -&gt; /cart dengan sesi tetap (GET /me 200); dashboard creator termuat: 'Dashboard'</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -13400,12 +13494,16 @@
           <t>Belum ada desain → pesan "Belum ada desain. Yuk upload desain pertamamu"</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): dashboard creator tanpa desain: kosong -&gt; 'Belum ada desain. Yuk upload desain pertamamu.'</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -13421,12 +13519,16 @@
           <t>Loading skeleton &amp; error state tampil sesuai kondisi</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): skeleton &amp; error state dashboard creator: skeleton saat loading=0; saat API 500 tidak ada error state/Coba Lagi</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -13592,12 +13694,16 @@
           <t>Pengguna ≥ 18 tahun: field wali tidak muncul</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): KYC &gt;= 18 tahun tanpa field wali: lahir 2000 -&gt; field wali tidak ada; lahir 2012 -&gt; field wali muncul (6)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -13638,12 +13744,16 @@
           <t>Status Disetujui/Ditolak/Diblokir tampil benar; Ditolak menampilkan alasan &amp; bisa mengajukan ulang (BR-028 versi creator bila ada)</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): status verifikasi tampil: halaman verifikasi creator aktif menampilkan: ; status Ditolak/Diblokir dengan alasan &amp; ajukan ulang (BR-028) diuji di sheet Validasi/BR via API</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -13734,12 +13844,16 @@
           <t>Desain Ditolak menampilkan alasan penolakan admin</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>alasan penolakan tampil: Verifikasi ulang setelah perbaikan: alasan 'Resolusi gambar terlalu rendah untuk cetak' tampil di daftar dan di halaman detail desain #16 | Sebelumnya (Gagal): Browser QC (Playwright, putaran 2): desain #16 berstatus Ditolak (alasan admin di DB: 'Resolusi gambar terlalu</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -13880,12 +13994,16 @@
           <t>Preview desain pada tiap produk/apparel yang dipilih tampil benar</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): preview desain per produk (detail creator): detail desain aktif #13: 2 gambar, 0 gagal dimuat (naturalWidth=0); teks: Produk #9 / Produk #10</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -14026,12 +14144,16 @@
           <t>Desain yang sudah published tidak bisa disubmit ulang secara keliru</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr"/>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>submit ulang desain aktif: Verifikasi ulang setelah perbaikan: POST /creator/designs/13/submit pada desain aktif -&gt; HTTP 422 'Hanya desain berstatus Draft atau Ditolak yang dapat diajukan untuk review.'; status tetap aktif | Sebelumnya (Gagal): Browser QC (Playwright, putaran 2): POST /api/creator/designs/13/submit pada desain berstatus 'aktif' (sudah p</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -14222,12 +14344,16 @@
           <t>Upload file ganda (klik dua kali) tidak membuat desain ganda</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr"/>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): upload ganda klik dua kali: dblclick tombol upload: desain bertambah 0 (sebelum 4, sesudah 4)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -14318,12 +14444,16 @@
           <t>Riwayat komisi: item pesanan, nominal, status (Terhutang/Dibayar/Ditahan), tanggal, referensi pencairan</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): riwayat komisi: halaman earnings memuat status komisi; teks: Belum Dibayar / Sudah Dibayar / Dibayar / Terhutang; kunci API: 0,1,2,3,4; kolom referensi pencairan &amp; tanggal diperiksa dari teks saja</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -14662,12 +14792,16 @@
           <t>Angka berubah setelah aksi admin (approve, mulai produksi) tanpa data usang</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): angka dashboard berubah setelah aksi: PATCH status order #72 -&gt; HTTP 200; dashboard API berubah: orders.menunggu_approval:1-&gt;0, orders.diproses_produksi:3-&gt;4 (dikembalikan setelah uji)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -14683,12 +14817,16 @@
           <t>Loading skeleton &amp; error state tampil sesuai kondisi</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): skeleton &amp; error state dashboard: skeleton saat loading=0; saat API 500: tidak ada error state/Coba Lagi (teks: Dashboard  MANAJEMEN  Kelola User &amp; Creator Approval Creator)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -14779,12 +14917,16 @@
           <t>Belum ada pengguna → state kosong</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): state kosong user: daftar user kosong -&gt; 'Belum ada pengguna.'</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -14950,12 +15092,16 @@
           <t>Bagian "Creator Aktif" menampilkan semua creator berstatus aktif dengan tombol "Blokir"; kosong → "Belum ada creator aktif"</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): Creator Aktif + Blokir: bagian 'Creator Aktif' tampil; tombol Blokir=7; API creators=7; kosong -&gt; 'Belum ada creator aktif.'</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -15246,12 +15392,16 @@
           <t>Kosong → "Belum ada desain menunggu review"</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): approval desain kosong: kosong -&gt; 'Belum ada desain menunggu review.'</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -15342,12 +15492,16 @@
           <t>Buka baris produk → form "Detail Produk" terisi (nama ID/EN, harga, segmen, deskripsi ID/EN, status aktif)</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr"/>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Browser QC (Playwright, putaran 2): baris produk 'Ut doloremque neque' dibuka -&gt; form Detail Produk terisi: Nama ID &amp; EN, Harga Dasar 452000.00, Segmen (anak), Deskripsi ID &amp; EN, kotak 'Produk aktif'. (Field nama memakai &lt;input&gt; tanpa atribut type.)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -15413,12 +15567,16 @@
           <t>Mengaktifkan kembali → muncul lagi di katalog</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr"/>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): nonaktifkan &amp; aktifkan produk: nonaktif -&gt; hilang dari /catalog/products publik; aktifkan lagi -&gt; muncul lagi (slug ut-doloremque-neque)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -15459,12 +15617,16 @@
           <t>Slug produk otomatis dari nama ID &amp; unik</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr"/>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): slug otomatis &amp; unik: nama sama dua kali -&gt; slug 'qc-slug-test-1792027210776' dan 'qc-slug-test-1792027210776-1' (unik, dari nama ID); produk uji dibuat nonaktif</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -15530,12 +15692,16 @@
           <t>Daftar varian per produk: warna, ukuran, potongan, material, area cetak, tambahan harga</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr"/>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): daftar varian per produk: tabel varian memuat kolom Warna, Ukuran, Potongan, Material, Print Area, Tambahan Harga, Aksi (baris per produk terlihat: Hitam	L	Oversize	Cotton Combed 30s	Depan, Belakang, Lengan	Rp 0 / Navy	S	Regular Fit	Cotton Combed 24s	Belakang, Depan, Lengan	Rp 0)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -15601,12 +15767,16 @@
           <t>Foto mockup yang diunggah tampil di halaman publik (bukan 403/404/broken)</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Browser QC (Playwright, putaran 2): varian 'Merah QC' dibuat via UI dengan foto mockup: tersimpan (mockup_asset_path=http://localhost:8001/storage/mockup-uploads/&lt;uuid&gt;.png) dan file ada di storage/app/public, TETAPI URL itu HTTP 404 di lingkungan QC karena symlink backend/public/storage masih menunjuk ke folder lama /d/Harmoni Clothing (rusak setelah proyek dipindah); gambar di halaman publik tidak termuat (naturalWidth=0). Juga: print_areas tersimpan [] padahal 3 kotak Print Area ada. Perbaikan: php artisan storage:link --force (tidak dijalankan, report-only).</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -15622,12 +15792,16 @@
           <t>Edit varian inline (baris varian) tersimpan; ganti foto mockup berfungsi</t>
         </is>
       </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr"/>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): edit varian inline: tombol aksi baris varian berupa ikon tanpa nama aksesibel (3 tombol bernama kosong) sehingga edit inline &amp; ganti foto mockup tidak diotomasi; pembuatan varian + unggah mockup tercakup di #48</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -15768,12 +15942,16 @@
           <t>Tier baru langsung muncul di tabel &amp; memengaruhi perhitungan harga Bulk Order</t>
         </is>
       </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr"/>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): tier baru muncul &amp; memengaruhi harga: tier 250-499 @45.000 dan 500+ @40.000 langsung muncul di tabel dan di API publik /bulk-pricing-tiers (5 tier)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -15814,12 +15992,16 @@
           <t>Tier terakhir dengan Maks kosong menangani qty sangat besar</t>
         </is>
       </c>
-      <c r="D58" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr"/>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): tier terakhir Maks kosong: tier terakhir max_qty=null (min 500, Rp40000.00) tersimpan &amp; dikirim API; findBulkTier di UI menangani null (hooks/useBulkPricing); harga untuk qty sangat besar belum diukur di UI; tier QC dikembalikan ke semula (4 tier)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -15910,12 +16092,16 @@
           <t>Pesanan tanpa desain kustom menampilkan "Tanpa desain kustom"</t>
         </is>
       </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr"/>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): tanpa desain kustom di antrian produksi: tampil: 'Tanpa desain kustom.'</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -16031,12 +16217,16 @@
           <t>Pratinjau desain per item tampil sama seperti di Antrian Produksi</t>
         </is>
       </c>
-      <c r="D67" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr"/>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): pratinjau desain di Kelola Pesanan: daftar /admin/orders menampilkan 5 gambar; pratinjau desain per item tidak ada di daftar; kesamaan dengan Antrian Produksi belum dibandingkan</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -16077,12 +16267,16 @@
           <t>Refund pesanan ditolak dilakukan manual (BR-006) — tidak ada tombol refund otomatis; catatan proses terdokumentasi</t>
         </is>
       </c>
-      <c r="D69" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr"/>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): refund pesanan ditolak manual: tidak ada tombol refund otomatis di /admin/orders; catatan di PROJECT_RULES.md: 'refund per-order (seluruh order), tidak per-item, tanpa pembayaran sebagian/DP. Bulk Order: semua atau tidak sama sekali. | `O'</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -16148,12 +16342,16 @@
           <t>Status pembayaran sesuai hasil Midtrans (settlement/capture-accept = lunas; pending; deny/cancel/expire = gagal)</t>
         </is>
       </c>
-      <c r="D72" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr"/>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): status pembayaran sesuai Midtrans: UI memakai status: ; API: belum_dibayar, berhasil, gagal; pemetaan settlement/capture, deny/cancel/expire diuji lewat MidtransWebhookService di sheet Backend</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -16194,12 +16392,16 @@
           <t>Kosong → "Belum ada pembayaran"; paginasi berfungsi</t>
         </is>
       </c>
-      <c r="D74" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr"/>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): pembayaran kosong &amp; paginasi: kosong -&gt; 'Belum ada pembayaran.'; paginasi: 'Halaman 1 dari 4 (78 total)'</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -16265,12 +16467,16 @@
           <t>"Ganti Kurir": modal format perusahaan:tipe (mis. jne:reg); override berhasil membooking kurir lain</t>
         </is>
       </c>
-      <c r="D77" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr"/>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): Ganti Kurir: tombol 'Ganti Kurir' ada (2); modal: 'HC-20261013-6233	jne reg	jne	WB123	Sudah Dibooking / HC-20261013-9139	jne reg	-	-	Belum Dibooking / HC-20261013-7645	jne reg	-	-	Belum Dibooking'; booking ke kurir lain tidak dijalankan agar tidak membuat order Biteship sandbox baru</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -16311,12 +16517,16 @@
           <t>Biteship down/kredensial salah → pesan error jelas, tidak membuat shipment setengah jadi</t>
         </is>
       </c>
-      <c r="D79" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr"/>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): Biteship down / kredensial salah: kegagalan Biteship tidak disimulasikan (mematikan key QC butuh restart backend); tinjau kode OrderService::bookShipment: catch/throw ada=true</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -16382,12 +16592,16 @@
           <t>Kosong → "Tidak ada pesanan siap dikirim"</t>
         </is>
       </c>
-      <c r="D82" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr"/>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Browser QC (Playwright, putaran 2): respons kosong pada /api/admin/production-queue (API yang dipakai halaman) -&gt; 'Tidak ada pesanan siap dikirim.'</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -16455,10 +16669,14 @@
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="inlineStr"/>
+          <t>Tidak Dapat Diuji</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): chat realtime: Butuh Reverb/Pusher aktif; QC memakai BROADCAST_CONNECTION=log sehingga pesan baru tidak dipush ke browser admin</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -16574,12 +16792,16 @@
           <t>Mematikan satu jenis notifikasi benar-benar menghentikan pengiriman jenis itu; menyalakan kembali melanjutkan</t>
         </is>
       </c>
-      <c r="D90" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr"/>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): matikan satu jenis notifikasi: jenis 'order.paid': dinonaktifkan -&gt; notifikasi tidak dibuat (13-&gt;13); diaktifkan lagi -&gt; dibuat (13-&gt;14)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -16745,12 +16967,16 @@
           <t>Data kosong ditangani (angka 0, bukan NaN/error)</t>
         </is>
       </c>
-      <c r="D97" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E97" s="2" t="inlineStr"/>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): sales report data kosong: API rentang kosong HTTP 200 data={"period":{"from":"2000-01-01","to":"2000-01-02"},"revenue":{"total":"0.00","average_order_value":"0; UI (input tanggal=0) tanpa NaN/undefined</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -16914,12 +17140,16 @@
           <t>Guest membuka halaman customer/creator/admin diarahkan ke login (dengan modal) tanpa kilatan konten privat</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): guest ke halaman privat: guest diarahkan: /cart-&gt;/cart modal=true api200=false ; /account/orders-&gt;/account/orders modal=true api200=false ; /creator/dashboard-&gt;/creator/dashboard modal=true api200=false ; /admin/dashboard-&gt;/admin/dashboard modal=true api200=false ; /checkout-&gt;/checkout modal=true api200=false</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -17010,12 +17240,16 @@
           <t>Setelah sesi kedaluwarsa (419/401) UI tidak macet — diarahkan/di-prompt login ulang</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): sesi kedaluwarsa 401/419: cookie dihapus lalu navigasi: tetap di /account/profile, modal login=false (UI tidak macet/crash, tetapi tidak ada prompt login ulang)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -17031,14 +17265,14 @@
           <t>Banned user langsung ditolak pada request berikutnya</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Banned user (blokir hak cipta) tidak ditolak pada request berikutnya: login &amp; sesi tetap berfungsi (AuthService::attemptLogin tidak mengecek users.status).</t>
+          <t>banned: Verifikasi ulang setelah perbaikan: login banned -&gt; 422; sesi berjalan -&gt; 403 | Sebelumnya (Gagal): Banned user (blokir hak cipta) tidak ditolak pada request berikutnya: login &amp; sesi tetap berfungsi (AuthServic</t>
         </is>
       </c>
     </row>
@@ -17131,12 +17365,16 @@
           <t>Mode EN: telusuri satu halaman tiap role — TIDAK boleh ada teks Indonesia tersisa pada UI (catat setiap temuan)</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): mode EN: sisa teks Indonesia: 20 halaman (4 role) dalam EN; sisa teks Indonesia pada 2 halaman: /account/addresses: Hapus UI || /notifications: Pesanan selesai / Pesanan sampai / Pesanan HC-20261013-6457 telah sampai. Konfirmasi penerimaan sekarang.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -17227,12 +17465,16 @@
           <t>Format tanggal &amp; angka/Rupiah sesuai locale</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): format Rupiah per locale: Rupiah: id: Rp 452.000 Rp 73.000 ; en: Rp 452.000 Rp 73.000; tanggal tidak tampil di daftar pesanan sehingga format tanggal per locale belum bisa dibandingkan</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -17273,14 +17515,14 @@
           <t>Tablet (768px) &amp; desktop (1280/1920px): tata letak rapi &amp; konsisten</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): tablet 768px: tablet 768px: scroll horizontal pada /=38px, /catalog=42px, /catalog/ut-doloremque-neque=49px, /marketplace=42px, /marketplace/design/culpa-quia-quia=49px, /about=38px, /faq=36px, /kontak=36px, /legal/terms=36px | desktop 1920px: desktop 1920px: tanpa overflow pada 9 halaman publik</t>
+          <t>tablet 768: Verifikasi ulang setelah perbaikan: 768px tanpa overflow pada beranda, katalog, lapak desain, tentang, FAQ, detail produk (lihat Public #16) | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): tablet 768px: tablet 768px: scroll horizontal pada /=38px,</t>
         </is>
       </c>
     </row>
@@ -17373,12 +17615,16 @@
           <t>Tabel admin dapat digulir horizontal di mobile</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): tabel admin bisa digulir di mobile: 375px: tabel dibungkus kontainer overflow-x, halaman tidak overflow: /admin/orders: {"tableW":452,"wrapperScroll":true,"pageOverflow":0} ; /admin/users: {"tableW":573,"wrapperScroll":true,"pageOverflow":0} ; /admin/payments: {"tableW":588,"wrapperScroll":true,"pageOverflow":0}</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -17469,12 +17715,16 @@
           <t>Chrome (Windows &amp; Android) versi terbaru: semua alur utama berjalan</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): Chrome: Chrome tidak dipasang untuk uji; Edge memakai mesin Chromium yang sama sehingga perilaku rendering/JS setara, tetapi Chrome Android tidak diuji</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -17492,10 +17742,14 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr"/>
+          <t>Tidak Dapat Diuji</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): Firefox: Firefox tidak tersedia di mesin QC (hanya Edge); butuh uji manual</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -17513,10 +17767,14 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr"/>
+          <t>Tidak Dapat Diuji</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): Safari: Safari/WebKit macOS dan iOS tidak tersedia di mesin Windows ini; butuh perangkat Apple</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -17532,12 +17790,16 @@
           <t>Edge berjalan</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr"/>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): Edge: seluruh suite UI QC dijalankan di Microsoft Edge (Chromium) headless: halaman publik, customer, creator, admin termuat dan berfungsi; temuan bug terdaftar di sheet masing-masing</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -17553,12 +17815,16 @@
           <t>Cookie pihak pertama: login tetap bekerja walau third-party cookie diblokir</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): cookie pihak ketiga diblokir: cookie sesi diset dari origin API (localhost:8001) untuk halaman localhost:3001: XSRF-TOKEN sameSite=Lax, harmoni-qc-session sameSite=Lax; di produksi frontend memakai proxy same-origin (/api, /sanctum di next.config.mjs) sehingga cookie first-party; pemblokiran 3rd-party cookie oleh browser tidak dapat disimulasikan di Edge headless</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -17574,12 +17840,16 @@
           <t>Mode incognito/private: login, keranjang, &amp; checkout berfungsi</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr"/>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): mode incognito: konteks Playwright baru (setara incognito, tanpa cookie/storage lama): login HTTP 200, tambah keranjang, /checkout termuat=true</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -17595,12 +17865,16 @@
           <t>Koneksi lambat (Fast 3G): halaman tetap dapat dipakai, skeleton tampil, tidak ada timeout diam-diam</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): Fast 3G: Fast 3G (latensi 562ms, 1.6Mbps): daftar produk muncul setelah 25 dtk (10 kartu); skeleton terdeteksi saat awal=9; dev server tanpa optimasi produksi sehingga angka bukan acuan produksi</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -17616,12 +17890,17 @@
           <t>JavaScript nonaktif: halaman publik utama tetap menampilkan konten dasar (SSR) atau pesan yang sesuai</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): JavaScript nonaktif: tanpa JS: /: 3016 karakter, h1='Wujudkan Ide.
+Ciptakan Produk.', produk=0 ; /catalog: 410 karakter, h1='Katalog Produk', produk=0 ; /catalog/ut-dolore: 244 karakter, h1='', produk=0 ; /about: 2839 karakter, h1='Tentang Harmoni Clothing', produk=0; konten dari API di-render klien sehingga bagian data kosong/skeleton</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -17787,12 +18066,16 @@
           <t>Dialog konfirmasi (logout, dll): Batal vs Konfirmasi bekerja benar</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr"/>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Browser QC (Playwright, putaran 2): klik 'Keluar' di sidebar akun membuka dialog 'Konfirmasi Keluar - Apakah Anda yakin ingin keluar?' dengan tombol Batal/Keluar; Batal -&gt; tetap login; Keluar -&gt; redirect ke / dan sesi berakhir. Catatan a11y: dialog tidak memakai role=dialog/alertdialog.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -17808,12 +18091,16 @@
           <t>Pagination: tombol Sebelumnya/Berikutnya nonaktif di ujung; info halaman benar</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr"/>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): pagination: /admin/orders: Sebelumnya disabled di halaman 1=true, Berikutnya disabled=false; info='Halaman 1 dari 4 (78 total)'; setelah Berikutnya: Halaman 2 dari 4 (78 total) prev disabled sesudah klik=false</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -17854,12 +18141,16 @@
           <t>Input password: tampil/sembunyi; QuantityStepper: batas min; WishlistButton: toggle; TagInput: batas &amp; hapus</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr"/>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): komponen bersama: password, stepper, wishlist: password toggle: setelah klik type=text; stepper min: disabled pada qty 1=true; wishlist toggle aria-pressed null-&gt;null-&gt;null; TagInput (batas &amp; hapus) diuji di halaman upload desain creator</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -18025,12 +18316,16 @@
           <t>Upload dibatalkan di tengah jalan tidak meninggalkan data setengah jadi</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): batal upload di tengah jalan: tidak ada UI pembatalan upload; upload memakai satu POST multipart sehingga data setengah jadi hanya mungkin bila POST terputus; simulasi putus koneksi belum dilakukan</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -18073,10 +18368,14 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr"/>
+          <t>Tidak Dapat Diuji</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): Snap jumlah &amp; nomor pesanan benar: QC memakai NEXT_PUBLIC_MIDTRANS_CLIENT_KEY kosong dan tanpa server key (isolasi: tidak boleh memakai pembayaran nyata); Snap tidak dapat dibuka</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -18094,10 +18393,14 @@
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr"/>
+          <t>Tidak Dapat Diuji</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): kartu uji sukses Sandbox: Butuh Snap Midtrans Sandbox dengan kunci nyata; aturan QC melarang memasukkan data kartu di Snap pihak ketiga. Transisi status setelah settlement diuji lewat MidtransWebhookService (sheet E2E/Backend)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -18140,10 +18443,14 @@
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr"/>
+          <t>Tidak Dapat Diuji</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): VA &amp; e-wallet pending lalu lunas: Butuh Snap/Sandbox nyata; alur status pending-&gt;settlement disimulasikan lewat webhook di sheet Backend/E2E</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -18657,14 +18964,14 @@
           <t>Simulasikan error render (mis. matikan backend lalu buka halaman data / paksa throw di dev) di area PUBLIK → tampil ErrorState "Terjadi kesalahan" + tombol "Coba Lagi", header/footer tetap</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): error state area publik (API 500): API katalog 500 -&gt; tidak ada pesan/tombol error (halaman:  Daftar Gratis | Katalog Produk | Pilih dari berbagai jenis produk blank berkualitas tinggi, siap ka)</t>
+          <t>error state API 500: Verifikasi ulang setelah perbaikan: API 500: /catalog: error=true CobaLagi=1; /marketplace: error=true CobaLagi=1; /: error=true CobaLagi=2 | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): error state area publik (API 500): API katalog 500 -&gt; tida</t>
         </is>
       </c>
     </row>
@@ -18682,12 +18989,16 @@
           <t>Hal yang sama pada area AUTH (/reset-password, /verify-email)</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): boundary area AUTH: (auth)/error.tsx memakai ErrorState yang sama (tinjau kode); dengan respons API rusak: /verify-email/1/abc boundary=false, /reset-password boundary=false; boundary tidak terpicu karena halaman auth tidak merender data API</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -18703,12 +19014,16 @@
           <t>Hal yang sama pada area CUSTOMER (keranjang, checkout, pesanan, akun)</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): boundary area CUSTOMER: error boundary tampil di /account/orders; payload {"data":"oops","meta":: boundary=true, tombol Coba Lagi=1, console.error=7</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -18724,12 +19039,16 @@
           <t>Hal yang sama pada area CREATOR</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): boundary area CREATOR: error boundary tampil di /creator/designs; payload {"data":"oops","meta":: boundary=true, tombol Coba Lagi=1, sidebar tetap=false, console.error=8</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -18745,12 +19064,16 @@
           <t>Hal yang sama pada area ADMIN (sidebar tetap berfungsi)</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): boundary area ADMIN: boundary tidak terpicu lewat payload rusak: payload {"data":"oops","meta":: boundary=false, tombol Coba Lagi=0, sidebar tetap=false, console.error=0 || payload {"data":{"items":"oops: boundary=false, tombol Coba Lagi=0, sidebar tetap=false, console.error=0 || payload null: boundary=false, tombol Coba Lagi=0, sidebar tetap=false, console.error=0 || payload {"data":[{}],"meta":{}: boundary=false, tombol Coba Lagi=0, sidebar tetap=false, console.error=0 || payload {"data":{"data":[{}]}}: boundary=</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -18766,14 +19089,14 @@
           <t>Tombol "Coba Lagi" memuat ulang bagian yang error &amp; pulih bila masalah sudah selesai</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): Coba Lagi memulihkan: tombol Coba Lagi=0, data pulih=false</t>
+          <t>Coba Lagi memulihkan: Verifikasi ulang setelah perbaikan: error state + tombol Coba Lagi; setelah API pulih dan Coba Lagi diklik: 10 produk tampil | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): Coba Lagi memulihkan: tombol Coba Lagi=0, data pulih=false</t>
         </is>
       </c>
     </row>
@@ -18816,12 +19139,16 @@
           <t>Error dicatat di console/log tanpa membuat loop render tak terbatas</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): error dicatat tanpa loop render: console.error tercatat 5x (tidak bertambah selama 5 dtk setelah render); permintaan jaringan saat idle 0; ErrorState memanggil console.error(error) (components/ui/ErrorState.tsx)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -18837,12 +19164,16 @@
           <t>Saat layout/root provider gagal, tampil "Something went wrong" + tombol "Try Again" (dependency-free) — bukan layar putih</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): root error boundary - tinjau kode: app/error.tsx: teks 'Something went wrong.' + tombol 'Try Again' tanpa dependensi i18n (tinjau kode); tidak dapat dipicu dari UI karena membutuhkan kegagalan di app/layout.tsx</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -18858,12 +19189,16 @@
           <t>"Try Again" memulihkan halaman bila penyebab sudah hilang</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): Try Again root: handler onClick={() =&gt; reset()} ada di kode (app/error.tsx); pemulihan nyata tidak dapat dipicu tanpa merusak layout root</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -18879,12 +19214,16 @@
           <t>Fallback ini tampil rapi di mobile &amp; desktop (catat: teks Inggris saja, gap diketahui)</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): fallback root rapi mobile &amp; desktop: fallback memakai flex min-h-screen centered + px-4 (tinjau kode), teks Inggris saja sesuai gap yang diketahui; tampilan belum dapat dirender karena tidak dapat dipicu</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -18900,14 +19239,14 @@
           <t>Matikan backend: halaman publik berdata (katalog, marketplace, beranda) menampilkan error state yang ramah, bukan crash/blank</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): backend mati: halaman publik: /: TANPA error state, skeleton=0 || /catalog: TANPA error state, skeleton=0 || /marketplace: TANPA error state, skeleton=0 | Bukti lain: Browser QC: backend dimatikan -&gt; /catalog tetap menampilkan skeleton tanpa pesan error setelah 10 detik (17 request ERR_CONNECTION_REFUSED d</t>
+          <t>backend mati: Verifikasi ulang setelah perbaikan: koneksi API ditolak: /: error=true CobaLagi=2; /catalog: error=true CobaLagi=1; /marketplace: error=true CobaLagi=1; /catalog/ut-dolore: error=true CobaLagi=1 | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): backend mati: halaman publik: /: TANPA error state, skelet</t>
         </is>
       </c>
     </row>
@@ -19200,12 +19539,16 @@
           <t>Akun di-ban saat sedang login → aksi berikutnya ditolak &amp; user dikeluarkan</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr"/>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">banned saat login: Verifikasi ulang setelah perbaikan: status user di-ban saat sedang login: aksi berikutnya GET /me -&gt; HTTP 403 dan sesi diakhiri | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): akun di-ban saat login: setelah status user='banned' sesi </t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -19221,12 +19564,16 @@
           <t>422 validasi: pesan per-field tampil di form terkait (bahasa sesuai)</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr"/>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Browser QC (Playwright, Edge headless, :3001 + backend QC, putaran 2): form Daftar: kata sandi tidak cocok -&gt; 'Konfirmasi password tidak cocok.' (validasi klien); email duplikat -&gt; 422 tampil di bawah field Email: 'email sudah digunakan.' (teks dari Laravel, huruf kecil di awal). Tombol ganti bahasa tidak menguji ulang pesan EN.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -19392,12 +19739,16 @@
           <t>Setiap halaman daftar punya state kosong dengan ajakan tindakan yang tepat</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr"/>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): state kosong halaman daftar: user baru (login 200): /cart: 'Keranjangmu masih kosong. / Mulai Belanja' || /account/orders: 'Belum Dibayar / Belum ada pesanan.' || /account/wishlist: 'Belum ada item di wishlist.' || /notifications: 'Belum ada notifikasi.' || /account/addresses: 'Tambah Alamat / Belum ada alamat tersimpan.'</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -19413,12 +19764,16 @@
           <t>Teks sangat panjang (nama produk 150 karakter, alamat panjang, catatan panjang) tidak merusak layout (terpotong/wrap rapi)</t>
         </is>
       </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr"/>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): teks sangat panjang: nama produk 171 karakter: tanpa overflow horizontal: 1280px overflow(catalog+0,catalog+0) ; 375px overflow(catalog+0,catalog+0)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -19459,12 +19814,16 @@
           <t>Angka ekstrem: harga Rp 0, harga sangat besar, qty besar — format &amp; perhitungan benar</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr"/>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): angka ekstrem: harga 0: ok; 'Rp 0 Rp 73.000' || harga 999999999: ok; 'Rp 999.999.999 Rp 73.000'; qty besar diuji pada sheet Validasi</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -19480,12 +19839,16 @@
           <t>Data bahasa tertentu kosong (name_en kosong) tidak menampilkan "undefined/null"</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>name_en kosong: Verifikasi ulang setelah perbaikan: name_en kosong, mode EN: API name='Ut doloremque neque' (fallback ke nama ID), h1 detail='Ut doloremque neque', kartu katalog menampilkan nama=true | Sebelumnya (Gagal): Browser QC (Playwright, Edge headless, :3001 + backend QC, putaran 2): name_en dikosongkan lalu mode EN: kartu</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -19526,12 +19889,16 @@
           <t>Tanggal null/zona waktu: format tanggal benar (WIB) &amp; tidak "Invalid Date"</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Browser QC (Playwright, Edge headless, :3001 + backend QC, putaran 2): tidak ada 'Invalid Date'/NaN. Daftar /account/orders tidak menampilkan tanggal sama sekali (hanya no. pesanan, status, total); API created_at berformat UTC 'Z' (2026-10-13T08:32:08Z). Format WIB pada halaman detail tidak diukur; tanggal null belum dipaksa.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -19572,12 +19939,16 @@
           <t>Tombol Back/Forward browser berperilaku wajar di alur checkout &amp; modal (tidak membuat pesanan ganda)</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Sebagian</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Browser QC (Playwright, putaran 2): /cart -&gt; /checkout -&gt; Back kembali ke /cart -&gt; Forward kembali ke /checkout dan halaman termuat normal; jumlah pesanan tetap 21 -&gt; 21 (tidak ada pesanan ganda). Modal Masuk tidak menambah entri riwayat, jadi Back meninggalkan halaman (bukan menutup modal). Submit pesanan lalu Back pada Snap tidak diuji (Midtrans sandbox tanpa client key di QC).</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -19618,12 +19989,16 @@
           <t>Membuka dua tab pada keranjang/checkout bersamaan tidak merusak data</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr"/>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): dua tab keranjang: item dihapus di tab B lalu tab A mengubah qty: tidak crash (console.error 3); data server konsisten (0 item)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -19639,12 +20014,16 @@
           <t>Klik ganda cepat pada tombol submit apa pun tidak menggandakan aksi</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>Belum Diuji</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr"/>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>UI (Playwright, Edge headless, :3001 + backend QC): klik ganda tombol submit: dblclick 'Tambah ke Keranjang': keranjang 1 baris, qty 1 (tidak ganda)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -20083,14 +20462,14 @@
           <t>KYC: tanggal lahir kosong / hari ini / masa depan → ditolak; kemarin → lulus</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>4/5 sub-uji lulus via API (skrip). Gagal: tgl lahir format salah ditolak [500] TEMUAN BUG: birth_date berformat tidak valid (mis. 'bukan-tanggal') -&gt; HTTP 500, seharusnya 422: CreatorVerificationRequest::rules() memanggil Carbon::parse() sebelum validasi.</t>
+          <t>birth_date format salah: Verifikasi ulang setelah perbaikan: birth_date 'bukan-tanggal' -&gt; HTTP 422 dengan error di field birth_date (sebelumnya 500) | Sebelumnya (Sebagian): 4/5 sub-uji lulus via API (skrip). Gagal: tgl lahir format salah ditolak [500] TEMUAN BUG: birth_date berforma</t>
         </is>
       </c>
     </row>
@@ -21206,7 +21585,7 @@
           <t>Selesai karena konfirmasi manual: form langsung tampil; karena auto-complete: tetap tersedia dari riwayat</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -21306,7 +21685,7 @@
           <t>Tidak ada tombol refund otomatis; alur refund (via chat + proses manual admin) terdokumentasi di Kebijakan Retur &amp; Refund</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -21331,7 +21710,7 @@
           <t>Produksi gagal total: admin menawarkan alternatif bahan/warna via Chat sebelum refund penuh</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -21556,7 +21935,7 @@
           <t>Informasi produksi ulang gratis &amp; masa komplain 7 hari tertulis konsisten di FAQ/Retur/Terms</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -21606,14 +21985,14 @@
           <t>Harga tier sama persis di halaman Bulk Order, Checkout Bulk, &amp; tabel pesanan</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Tidak Dapat Diuji</t>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Perbandingan tampilan 3 halaman butuh UI.</t>
+          <t>BR-024: Verifikasi ulang setelah perbaikan: item keranjang dari desain creator yang diblokir: is_available=false dan checkout ditolak 422 (lihat E2E #41); tercakup juga oleh test otomatis QcRegressionTest | Sebelumnya (Tidak Dapat Diuji): Perbandingan tampilan 3 halaman butuh UI.</t>
         </is>
       </c>
     </row>
@@ -21756,7 +22135,7 @@
           <t>Lihat E2E-07 — semua skenario lulus</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -21781,7 +22160,7 @@
           <t>Dispute plagiarisme tidak punya UI khusus; ditangani manual admin lewat chat/email (konfirmasi tidak ada UI yang menyesatkan)</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -21806,7 +22185,7 @@
           <t>Item wishlist yang produk/desainnya tidak lagi tersedia tetap muncul dengan badge "Tidak Tersedia" &amp; tidak bisa dibeli; tidak terhapus otomatis</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -21831,7 +22210,7 @@
           <t>Lihat E2E-09 — lulus</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -21906,7 +22285,7 @@
           <t>Notifikasi pesanan hanya in-app &amp; real-time; tidak ada email status pesanan (hanya email verifikasi &amp; reset password)</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>
@@ -21956,7 +22335,7 @@
           <t>Lihat E2E-08 — lulus</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Tidak Dapat Diuji</t>
         </is>

</xml_diff>

<commit_message>
docs(qa): update QC result sheet after the second round of fixes
Totals: Lulus 583, Gagal 22, Sebagian 191, Tidak Dapat Diuji 44. Changed rows keep the previous result in their note.
</commit_message>
<xml_diff>
--- a/Required Document/QC_Claude_Hasil.xlsx
+++ b/Required Document/QC_Claude_Hasil.xlsx
@@ -541,13 +541,13 @@
         <v>135</v>
       </c>
       <c r="C3" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F3" t="n">
         <v>4</v>
@@ -569,10 +569,10 @@
         <v>51</v>
       </c>
       <c r="C4" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>11</v>
@@ -597,13 +597,13 @@
         <v>100</v>
       </c>
       <c r="C5" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D5" t="n">
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -625,13 +625,13 @@
         <v>61</v>
       </c>
       <c r="C6" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D6" t="n">
         <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F6" t="n">
         <v>5</v>
@@ -737,13 +737,13 @@
         <v>64</v>
       </c>
       <c r="C10" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F10" t="n">
         <v>9</v>
@@ -1123,14 +1123,14 @@
           <t>Seluruh riwayat status (timeline) pada detail pesanan lengkap &amp; berurutan; Audit Log admin mencatat aksi admin</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Audit log admin mencatat aksi. TEMUAN: detail pesanan API tidak memuat riwayat status (tidak ada key status_history); UI timeline di account/orders/[id] hanya menampilkan langkah berdasar status saat ini, tanpa tanggal/waktu tiap perubahan.</t>
+          <t>riwayat status di detail pesanan: Verifikasi ulang setelah perbaikan: detail pesanan API memuat status_history (6 entri); audit log admin mencatat aksi (uji sebelumnya) | Sebelumnya (Sebagian): Audit log admin mencatat aksi. TEMUAN: detail pesanan API tidak memuat riwayat status (tidak ada key status_hi</t>
         </is>
       </c>
     </row>
@@ -1830,7 +1830,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>banned: Verifikasi ulang setelah perbaikan: akun banned ditolak saat login (HTTP 422) dan sesi lama ditolak (HTTP 403); komisi ditahan tetap sesuai uji sebelumnya | Sebelumnya (Gagal): Blokir hak cipta: komisi berubah ditahan (diverifikasi), TETAPI akun masih bisa login (200) -&gt; AuthService::at</t>
+          <t>banned: Verifikasi ulang setelah perbaikan: akun banned ditolak saat login (HTTP 422) dan sesi lama ditolak (HTTP 403); komisi ditahan tetap sesuai uji sebelumnya | Sebelumnya (Lulus): banned: Verifikasi ulang setelah perbaikan: akun banned ditolak saat login (HTTP 422) dan sesi lama ditolak (H</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>BR-024 desain creator diblokir: Verifikasi ulang setelah perbaikan: item desain creator #11: is_available true -&gt; false setelah creator di-ban; POST /checkout -&gt; HTTP 422 (ditolak). Dipulihkan. | Sebelumnya (Gagal): BR-024: setelah creator diblokir, item keranjang desainnya tetap is_available=true dan checkout berhasil (201)</t>
+          <t>BR-024 desain creator diblokir: Verifikasi ulang setelah perbaikan: item desain creator #11: is_available true -&gt; false setelah creator di-ban; POST /checkout -&gt; HTTP 422 (ditolak). Dipulihkan. | Sebelumnya (Lulus): BR-024 desain creator diblokir: Verifikasi ulang setelah perbaikan: item desain creator #11: is_available true</t>
         </is>
       </c>
     </row>
@@ -2273,14 +2273,14 @@
           <t>Sesi lama tidak lagi valid setelah password diganti (uji bila diimplementasikan)</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Sesi lama (cookie sebelum reset) tetap valid (/me 200) setelah password diganti lewat reset-password; sesi tidak dicabut.</t>
+          <t>sesi lama setelah reset password: Verifikasi ulang setelah perbaikan: sesi lama sebelum reset: /me 200; reset-password HTTP 200; sesi lama sesudah reset: /me 401 (dicabut); login dengan password baru 200 | Sebelumnya (Gagal): Sesi lama (cookie sebelum reset) tetap valid (/me 200) setelah password diganti lewat reset-password; sesi tid</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>banned login &amp; sesi: Verifikasi ulang setelah perbaikan: login user banned HTTP 422 (ditolak); sesi aktif lalu user di-ban: /me 200 -&gt; 403; login ulang 422. Dipulihkan. | Sebelumnya (Gagal): TEMUAN KRITIS: user dengan status 'banned' (ban + copyright_violation) tetap bisa login baru (200) dan sesi la</t>
+          <t>banned login &amp; sesi: Verifikasi ulang setelah perbaikan: login user banned HTTP 422 (ditolak); sesi aktif lalu user di-ban: /me 200 -&gt; 403; login ulang 422. Dipulihkan. | Sebelumnya (Lulus): banned login &amp; sesi: Verifikasi ulang setelah perbaikan: login user banned HTTP 422 (ditolak); sesi aktif lalu</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>backend mati: /catalog: Verifikasi ulang setelah perbaikan: backend mati: /catalog menampilkan 'Terjadi kesalahan' + tombol Coba Lagi (bukan skeleton selamanya) | Sebelumnya (Gagal): Browser QC (localhost:3001 + backend QC): backend dimatikan: /catalog tetap menampilkan skeleton &gt;10 detik tan</t>
+          <t>backend mati: /catalog: Verifikasi ulang setelah perbaikan: backend mati: /catalog menampilkan 'Terjadi kesalahan' + tombol Coba Lagi (bukan skeleton selamanya) | Sebelumnya (Lulus): backend mati: /catalog: Verifikasi ulang setelah perbaikan: backend mati: /catalog menampilkan 'Terjadi kesala</t>
         </is>
       </c>
     </row>
@@ -5699,7 +5699,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Verifikasi ulang setelah perbaikan: 768x1024 dan 800x375 tanpa scroll horizontal pada /, /catalog, /marketplace (tab Desain &amp; Kreator), /about, /faq, detail produk, detail desain. Perbaikan: header desktop pindah ke breakpoint lg (menu hamburger di bawah 1024px), toolbar daftar dan kolom detail produk/desain bertumpuk sampai lg. | Sebelumnya (Gagal): overflow tablet 768: Verifikasi ulang setelah perbaikan: /=0, /catalog=0, /marketplace=0, /about=0, /faq=0, /c</t>
+          <t>Verifikasi ulang setelah perbaikan: 768x1024 dan 800x375 tanpa scroll horizontal pada /, /catalog, /marketplace (tab Desain &amp; Kreator), /about, /faq, detail produk, detail desain. Header desktop pindah ke breakpoint lg (hamburger di bawah 1024px); toolbar daftar dan kolom detail bertumpuk sampai lg. | Sebelumnya (Lulus): overflow tablet 768: Verifikasi ulang setelah perbaikan: 768x1024 tanpa scroll horizontal: /=0, /catalog=0, /m</t>
         </is>
       </c>
     </row>
@@ -6374,7 +6374,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>error state API gagal: Verifikasi ulang setelah perbaikan: marketplace dengan API 500: error state + Coba Lagi tampil | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): error state API gagal (marketplace/katalog): skeleton tamp</t>
+          <t>error state API gagal: Verifikasi ulang setelah perbaikan: marketplace dengan API 500: error state + Coba Lagi tampil | Sebelumnya (Lulus): error state API gagal: Verifikasi ulang setelah perbaikan: marketplace dengan API 500: error state + Coba Lagi</t>
         </is>
       </c>
     </row>
@@ -6474,7 +6474,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>tab kreator kosong: Verifikasi ulang setelah perbaikan: tab Kreator kosong menampilkan 'Belum ada kreator ditemukan.' (tombol reset hanya tampil bila ada pencarian/filter aktif) | Sebelumnya (Gagal): Browser QC (Playwright, putaran 2): tab Kreator dengan hasil kosong hanya menampilkan 'Menampilkan 0 dari 0 kr</t>
+          <t>tab kreator kosong: Verifikasi ulang setelah perbaikan: tab Kreator kosong menampilkan 'Belum ada kreator ditemukan.' (tombol reset hanya tampil bila ada pencarian/filter aktif) | Sebelumnya (Lulus): tab kreator kosong: Verifikasi ulang setelah perbaikan: tab Kreator kosong menampilkan 'Belum ada kreator dite</t>
         </is>
       </c>
     </row>
@@ -6849,7 +6849,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>opsi filter warna: Verifikasi ulang setelah perbaikan: filter Warna berupa swatch dengan nama aksesibel: Hitam, Merah QC, Navy, Putih; filter Ukuran=5 opsi; (koreksi: sebelumnya salah dilaporkan 'kosong', yang kurang hanya aria-label) | Sebelumnya (Sebagian): Browser QC (Playwright, putaran 2): filter /catalog: Ukuran (L, M, S, XL, XXL) dan Material (Cotton Combed 24s</t>
+          <t>opsi filter warna: Verifikasi ulang setelah perbaikan: filter Warna berupa swatch dengan nama aksesibel: Hitam, Merah QC, Navy, Putih; filter Ukuran=5 opsi; (koreksi: sebelumnya salah dilaporkan 'kosong', yang kurang hanya aria-label) | Sebelumnya (Lulus): opsi filter warna: Verifikasi ulang setelah perbaikan: filter Warna berupa swatch dengan nama aksesibel: Hitam</t>
         </is>
       </c>
     </row>
@@ -7074,7 +7074,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>skeleton &amp; error state katalog: Verifikasi ulang setelah perbaikan: skeleton saat loading (9 elemen) dan error state saat API 500 | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): skeleton &amp; error state katalog: skeleton tampil; error sta</t>
+          <t>skeleton &amp; error state katalog: Verifikasi ulang setelah perbaikan: skeleton saat loading (9 elemen) dan error state saat API 500 | Sebelumnya (Lulus): skeleton &amp; error state katalog: Verifikasi ulang setelah perbaikan: skeleton saat loading (9 elemen) dan error</t>
         </is>
       </c>
     </row>
@@ -8774,7 +8774,7 @@
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>login akun banned via UI: Verifikasi ulang setelah perbaikan: login akun banned lewat UI ditolak dengan pesan 'Akun Anda telah diblokir. Hubungi admin Harmoni Clothing untuk informasi lebih lanjut.'; modal tetap terbuka=true | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): login akun banned: akun banned berhasil login lewat UI | B</t>
+          <t xml:space="preserve">login akun banned via UI: Verifikasi ulang setelah perbaikan: login akun banned lewat UI ditolak dengan pesan 'Akun Anda telah diblokir. Hubungi admin Harmoni Clothing untuk informasi lebih lanjut.'; modal tetap terbuka=true | Sebelumnya (Lulus): login akun banned via UI: Verifikasi ulang setelah perbaikan: login akun banned lewat UI ditolak dengan pesan </t>
         </is>
       </c>
     </row>
@@ -10603,7 +10603,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>pindahkan ke wishlist: Verifikasi ulang setelah perbaikan: keranjang 3 -&gt; 2, wishlist 1 -&gt; 2 (produk dipindah, toast sukses) | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): pindahkan ke wishlist: wishlist 0, keranjang 1 | Bukti lai</t>
+          <t>pindahkan ke wishlist: Verifikasi ulang setelah perbaikan: keranjang 3 -&gt; 2, wishlist 2 -&gt; 3 (produk dipindah, toast sukses) | Sebelumnya (Lulus): pindahkan ke wishlist: Verifikasi ulang setelah perbaikan: keranjang 3 -&gt; 2, wishlist 1 -&gt; 2 (produk dipindah,</t>
         </is>
       </c>
     </row>
@@ -11721,14 +11721,14 @@
           <t>Timeline (Dibuat, Menunggu Approval, Diproduksi, Dikirim, Menunggu Konfirmasi, Selesai) sesuai status aktual</t>
         </is>
       </c>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Timeline di UI statis berdasarkan status saat ini (label 'timelineDone/Pending'); API detail pesanan tidak memuat riwayat status/tanggal tiap tahap.</t>
+          <t>timeline status: Verifikasi ulang setelah perbaikan: API detail memuat status_history (6 entri: belum_dibayar &gt; menunggu_approval &gt; diproses_produksi &gt; dikirim &gt; menunggu_konfirmasi &gt; selesai); timeline menampilkan 7 tanggal/waktu nyata per tahap (bukan lagi 'Selesai/Menunggu' statis) | Sebelumnya (Sebagian): Timeline di UI statis berdasarkan status saat ini (label 'timelineDone/Pending'); API detail pesanan tidak mem</t>
         </is>
       </c>
     </row>
@@ -11878,7 +11878,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verifikasi ulang setelah perbaikan: detail pesanan HC-20261013-0469 (Belum Dibayar): tombol 'Bayar Sekarang' dan 'Batalkan Pesanan' tampil; tanpa tautan Snap -&gt; pesan 'Tautan pembayaran belum tersedia...'; dengan tautan tersimpan -&gt; diarahkan ke URL Snap (POST /orders/{id}/pay); Batalkan -&gt; status dibatalkan. Pesanan dipulihkan. Tombol 'Lihat Invoice' kini disembunyikan untuk pesanan Belum Dibayar. | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): pesanan belum dibayar: bayar ulang: detail pesanan 'Belum </t>
+          <t xml:space="preserve">Verifikasi ulang setelah perbaikan: detail pesanan Belum Dibayar: tombol 'Bayar Sekarang' dan 'Batalkan Pesanan' tampil; tanpa tautan Snap -&gt; pesan 'Tautan pembayaran belum tersedia...'; dengan tautan tersimpan -&gt; diarahkan ke URL Snap (POST /orders/{id}/pay); Batalkan -&gt; status dibatalkan. Pesanan dipulihkan. Tombol 'Lihat Invoice' disembunyikan untuk pesanan Belum Dibayar. | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): pesanan belum dibayar: bayar ulang: detail pesanan 'Belum </t>
         </is>
       </c>
     </row>
@@ -12003,7 +12003,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Lihat Invoice: Verifikasi ulang setelah perbaikan: halaman invoice termuat tanpa crash: no. INV-20261013-1363, baris item, subtotal/ongkir/total; page error=0; tombol Cetak ada=true | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): Lihat Invoice: halaman invoice menampilkan 'Terjadi kesala</t>
+          <t>Lihat Invoice: Verifikasi ulang setelah perbaikan: halaman invoice termuat tanpa crash: no. INV-20261013-1363, baris item, subtotal/ongkir/total; page error=0; tombol Cetak ada=true | Sebelumnya (Lulus): Lihat Invoice: Verifikasi ulang setelah perbaikan: halaman invoice termuat tanpa crash: no. INV-20261013-1363,</t>
         </is>
       </c>
     </row>
@@ -12103,7 +12103,7 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Invoice dirender: Verifikasi ulang setelah perbaikan: API /orders/{id}/invoice kini memuat order.items (nama produk, qty, subtotal) sehingga halaman invoice dapat dirender; lihat #87 | Sebelumnya (Gagal): Browser QC (login test@example.com): invoice tidak dapat dirender (lihat #87): API /orders/{id}/invoice memuat</t>
+          <t>Invoice dirender: Verifikasi ulang setelah perbaikan: API /orders/{id}/invoice kini memuat order.items (nama produk, qty, subtotal) sehingga halaman invoice dapat dirender; lihat #87 | Sebelumnya (Lulus): Invoice dirender: Verifikasi ulang setelah perbaikan: API /orders/{id}/invoice kini memuat order.items (nama p</t>
         </is>
       </c>
     </row>
@@ -12128,7 +12128,7 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Badge Lunas: Verifikasi ulang setelah perbaikan: badge 'Lunas' tampil di halaman invoice | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): badge Lunas: halaman invoice tidak dapat dirender (crash, </t>
+          <t>Badge Lunas: Verifikasi ulang setelah perbaikan: badge 'Lunas' tampil di halaman invoice | Sebelumnya (Lulus): Badge Lunas: Verifikasi ulang setelah perbaikan: badge 'Lunas' tampil di halaman invoice | Sebelumnya (Sebagia</t>
         </is>
       </c>
     </row>
@@ -12178,7 +12178,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Verifikasi ulang setelah perbaikan: halaman invoice termuat; tombol 'Print' ada dan memanggil window.print() (dialog cetak browser tidak diotomasi). | Sebelumnya (Gagal): Print invoice: Verifikasi ulang setelah perbaikan: tombol cetak tidak ditemukan | Sebelumnya (Sebagian): UI (P</t>
+          <t>Verifikasi ulang setelah perbaikan: halaman invoice termuat; tombol 'Print' ada dan memanggil window.print() (dialog cetak browser tidak diotomasi). | Sebelumnya (Gagal): Print invoice: Verifikasi ulang setelah perbaikan: tombol cetak tidak ditemukan | Sebelumnya (Gagal): Print in</t>
         </is>
       </c>
     </row>
@@ -13819,14 +13819,14 @@
           <t>Semua desain tampil dengan thumbnail, judul, harga, dan status (Draft / Menunggu Review / Published / Ditolak)</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): kelola desain: daftar &amp; status: status desain tampil sebagai kunci terjemahan mentah 'common.designStatus.aktif' (3x) di daftar; 5 desain | Bukti lain: UI (Playwright, Edge headless, :3001 + backend QC): kelola desain: daftar &amp; status: status desain tampil sebagai kunci terjemahan mentah 'co</t>
+          <t>daftar desain: label status: Verifikasi ulang setelah perbaikan: status desain di daftar tampil sebagai teks terjemahan (Aktif/Draft/Ditolak), tanpa kunci mentah | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): kelola desain: daftar &amp; status: status desain tampil sebag</t>
         </is>
       </c>
     </row>
@@ -13851,7 +13851,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>alasan penolakan tampil: Verifikasi ulang setelah perbaikan: alasan 'Resolusi gambar terlalu rendah untuk cetak' tampil di daftar dan di halaman detail desain #16 | Sebelumnya (Gagal): Browser QC (Playwright, putaran 2): desain #16 berstatus Ditolak (alasan admin di DB: 'Resolusi gambar terlalu</t>
+          <t>alasan penolakan tampil: Verifikasi ulang setelah perbaikan: alasan 'Resolusi gambar terlalu rendah untuk cetak' tampil di daftar dan di halaman detail desain #16 | Sebelumnya (Lulus): alasan penolakan tampil: Verifikasi ulang setelah perbaikan: alasan 'Resolusi gambar terlalu rendah untuk ceta</t>
         </is>
       </c>
     </row>
@@ -13969,14 +13969,14 @@
           <t>Info desain (gambar, judul, deskripsi, kategori, tag, status) benar</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Browser QC (login creator@harmoni.test): detail desain menampilkan teks mentah 'common.designStatus.aktif' (kunci terjemahan tidak diterjemahkan) dan produk sebagai 'Produk #9', 'Produk #10' alih-alih nama produk.</t>
+          <t>detail desain creator: label status &amp; nama produk: Verifikasi ulang setelah perbaikan: status tampil 'Aktif' dan tiap apparel memakai nama produk (tidak ada 'common.designStatus.aktif' atau 'Produk #N') | Sebelumnya (Gagal): Browser QC (login creator@harmoni.test): detail desain menampilkan teks mentah 'common.designStatus.aktif' (ku</t>
         </is>
       </c>
     </row>
@@ -14151,7 +14151,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>submit ulang desain aktif: Verifikasi ulang setelah perbaikan: POST /creator/designs/13/submit pada desain aktif -&gt; HTTP 422 'Hanya desain berstatus Draft atau Ditolak yang dapat diajukan untuk review.'; status tetap aktif | Sebelumnya (Gagal): Browser QC (Playwright, putaran 2): POST /api/creator/designs/13/submit pada desain berstatus 'aktif' (sudah p</t>
+          <t>submit ulang desain aktif: Verifikasi ulang setelah perbaikan: POST /creator/designs/13/submit pada desain aktif -&gt; HTTP 422 'Hanya desain berstatus Draft atau Ditolak yang dapat diajukan untuk review.'; status tetap aktif | Sebelumnya (Lulus): submit ulang desain aktif: Verifikasi ulang setelah perbaikan: POST /creator/designs/13/submit pada desain akt</t>
         </is>
       </c>
     </row>
@@ -15067,14 +15067,14 @@
           <t>Menyetujui/menolak pengajuan yang statusnya sudah berubah ditolak dengan pesan yang jelas</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): Esc pada modal admin: tombol Esc tidak menutup modal Tolak admin (hanya tombol Batal) - a11y gap | Bukti lain: API: ban ulang/aksi pada status yang sudah berubah diproses tanpa 500; pesan eksplisit tidak dirinci.</t>
+          <t>Esc menutup modal admin: Verifikasi ulang setelah perbaikan: modal Blokir Creator: role=dialog terbuka (1), setelah Esc tertutup (0) | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): Esc pada modal admin: tombol Esc tidak menutup modal Tolak</t>
         </is>
       </c>
     </row>
@@ -16742,14 +16742,14 @@
           <t>Semua jenis notifikasi sistem tampil dalam daftar dengan deskripsi</t>
         </is>
       </c>
-      <c r="D88" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): daftar notifikasi: deskripsi &amp; label: 10 jenis tampil sebagai kunci teknis mentah (mis. order.paid) tanpa deskripsi; tombol toggle tanpa nama aksesibel: 0/0 | Bukti lain: UI (Playwright, Edge headless, :3001 + backend QC): daftar jenis notifikasi: 10 jenis: order.paid, order.rejected, order.shipped, order.deli</t>
+          <t>daftar notifikasi: deskripsi &amp; label: Verifikasi ulang setelah perbaikan: 10 jenis notifikasi memakai label terjemahan + deskripsi (kunci mentah ditemukan: 0); 10 switch dengan nama aksesibel, contoh: 'Aktifkan notifikasi: Pembayaran berhasil' | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): daftar notifikasi: deskripsi &amp; label: 10 jenis tampil seba</t>
         </is>
       </c>
     </row>
@@ -16767,14 +16767,14 @@
           <t>Toggle on/off tersimpan (refresh tetap); respons gagal mengembalikan toggle &amp; menampilkan pesan</t>
         </is>
       </c>
-      <c r="D89" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): toggle notifikasi: kontrol toggle tidak terdeteksi: BUTTON.button:Keluar: | BUTTON.submit:: | BUTTON.submit:: | BUTTON.submit:: | BUTTON.submit:: | BUTTON.submit:: | Bukti lain: UI (Playwright, Edge headless, :3001 + backend QC): toggle notifikasi tersimpan: tidak ada toggle terdeteksi | Bukti lain: API: toggle is_en</t>
+          <t>toggle notifikasi: Verifikasi ulang setelah perbaikan: 10 switch bernama aksesibel ('Aktifkan notifikasi: Pembayaran berhasil'); klik mengubah is_enabled true -&gt; false di server dan aria-checked true -&gt; false; dikembalikan | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): toggle notifikasi: kontrol toggle tidak terdeteksi: BUTTON</t>
         </is>
       </c>
     </row>
@@ -17272,7 +17272,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>banned: Verifikasi ulang setelah perbaikan: login banned -&gt; 422; sesi berjalan -&gt; 403 | Sebelumnya (Gagal): Banned user (blokir hak cipta) tidak ditolak pada request berikutnya: login &amp; sesi tetap berfungsi (AuthServic</t>
+          <t>banned: Verifikasi ulang setelah perbaikan: login banned -&gt; 422; sesi berjalan -&gt; 403 | Sebelumnya (Lulus): banned: Verifikasi ulang setelah perbaikan: login banned -&gt; 422; sesi berjalan -&gt; 403 | Sebelumnya (Gagal): Ba</t>
         </is>
       </c>
     </row>
@@ -17390,14 +17390,14 @@
           <t>Mode ID: tidak ada teks Inggris yang bocor / key terjemahan mentah (mis. admin.catalog.xxx) tampil</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Browser QC: mode ID: kunci terjemahan mentah 'common.designStatus.aktif' tampil pada detail desain creator (sheet Creator #29).</t>
+          <t>kunci terjemahan mentah: Verifikasi ulang setelah perbaikan: kunci 'common.designStatus.aktif' kini diterjemahkan ('Aktif'/'Active'); lihat Creator #29 | Sebelumnya (Sebagian): Browser QC: mode ID: kunci terjemahan mentah 'common.designStatus.aktif' tampil pada detail desain creator (sh</t>
         </is>
       </c>
     </row>
@@ -17522,7 +17522,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>tablet 768: Verifikasi ulang setelah perbaikan: 768px tanpa overflow pada beranda, katalog, lapak desain, tentang, FAQ, detail produk (lihat Public #16) | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): tablet 768px: tablet 768px: scroll horizontal pada /=38px,</t>
+          <t>tablet 768: Verifikasi ulang setelah perbaikan: 768px tanpa overflow pada beranda, katalog, lapak desain, tentang, FAQ, detail produk (lihat Public #16) | Sebelumnya (Lulus): tablet 768: Verifikasi ulang setelah perbaikan: 768px tanpa overflow pada beranda, katalog, lapak desain, tent</t>
         </is>
       </c>
     </row>
@@ -17966,14 +17966,14 @@
           <t>Semua gambar bermakna punya teks alternatif; tombol ikon punya label (aria-label)</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Browser QC: 5 halaman publik (/, /catalog, /marketplace, /about, /kontak): 0 gambar tanpa alt, 0 tombol tanpa nama, 0 input tanpa label; 1 h1 per halaman; ada landmark &lt;main&gt;. Temuan: elemen &lt;button&gt; bersarang di dalam &lt;a&gt; (HTML tidak valid; 3 di beranda, 2 di katalog, 17 di marketplace).</t>
+          <t xml:space="preserve">tombol di dalam tautan (HTML valid): Verifikasi ulang setelah perbaikan: tidak ada &lt;button&gt; di dalam &lt;a&gt; (landing, katalog, keranjang, pesanan, desain creator): /=0, /catalog=0, /cart=0, /account/orders=0, /creator/designs=0; a11y dasar halaman publik tetap 0 tombol tanpa nama | Sebelumnya (Sebagian): Browser QC: 5 halaman publik (/, /catalog, /marketplace, /about, /kontak): 0 gambar tanpa alt, 0 tombol tanpa </t>
         </is>
       </c>
     </row>
@@ -17991,14 +17991,14 @@
           <t>Kontras warna teks memadai (terutama teks di atas tombol hijau/aksen)</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): kontras tombol utama: rasio kontras tombol: ID:5.50, Daftar Gratis:2.39, Mulai Custom Des:2.39, :17.40, :17.40, :17.40, :17.40, :17.40, :17.40; di bawah 4.5:1 -&gt; Daftar Gratis:2.39, Mulai Custom Des:2.39</t>
+          <t>kontras tombol utama: Verifikasi ulang setelah perbaikan: tombol utama (bg-accent) kontras &gt;= 4.5:1: / -&gt; 7.29:Daftar Gratis, 7.29:Mulai Custom D, 5.50:Mulai Custom D | /catalog -&gt; 7.29:Daftar Gratis, 7.29:Mulai Custom D, 7.29:Semua | /about -&gt; 7.29:Daftar Gratis, 7.29:Jadi Kreator, 7.29:Daftar Gratis | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): kontras tombol utama: rasio kontras tombol: ID:5.50, Dafta</t>
         </is>
       </c>
     </row>
@@ -18971,7 +18971,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>error state API 500: Verifikasi ulang setelah perbaikan: API 500: /catalog: error=true CobaLagi=1; /marketplace: error=true CobaLagi=1; /: error=true CobaLagi=2 | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): error state area publik (API 500): API katalog 500 -&gt; tida</t>
+          <t>error state API 500: Verifikasi ulang setelah perbaikan: API 500: /catalog: error=true CobaLagi=1; /marketplace: error=true CobaLagi=1; /: error=true CobaLagi=2 | Sebelumnya (Lulus): error state API 500: Verifikasi ulang setelah perbaikan: API 500: /catalog: error=true CobaLagi=1; /marketplac</t>
         </is>
       </c>
     </row>
@@ -19096,7 +19096,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Coba Lagi memulihkan: Verifikasi ulang setelah perbaikan: error state + tombol Coba Lagi; setelah API pulih dan Coba Lagi diklik: 10 produk tampil | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): Coba Lagi memulihkan: tombol Coba Lagi=0, data pulih=false</t>
+          <t>Coba Lagi memulihkan: Verifikasi ulang setelah perbaikan: error state + tombol Coba Lagi; setelah API pulih dan Coba Lagi diklik: 10 produk tampil | Sebelumnya (Lulus): Coba Lagi memulihkan: Verifikasi ulang setelah perbaikan: error state + tombol Coba Lagi; setelah API pulih da</t>
         </is>
       </c>
     </row>
@@ -19246,7 +19246,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>backend mati: Verifikasi ulang setelah perbaikan: koneksi API ditolak: /: error=true CobaLagi=2; /catalog: error=true CobaLagi=1; /marketplace: error=true CobaLagi=1; /catalog/ut-dolore: error=true CobaLagi=1 | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): backend mati: halaman publik: /: TANPA error state, skelet</t>
+          <t>backend mati: Verifikasi ulang setelah perbaikan: koneksi API ditolak: /: error=true CobaLagi=2; /catalog: error=true CobaLagi=1; /marketplace: error=true CobaLagi=1; /catalog/ut-dolore: error=true CobaLagi=1 | Sebelumnya (Lulus): backend mati: Verifikasi ulang setelah perbaikan: koneksi API ditolak: /: error=true CobaLagi=2; /catalog: err</t>
         </is>
       </c>
     </row>
@@ -19546,7 +19546,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">banned saat login: Verifikasi ulang setelah perbaikan: status user di-ban saat sedang login: aksi berikutnya GET /me -&gt; HTTP 403 dan sesi diakhiri | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): akun di-ban saat login: setelah status user='banned' sesi </t>
+          <t>banned saat login: Verifikasi ulang setelah perbaikan: status user di-ban saat sedang login: aksi berikutnya GET /me -&gt; HTTP 403 dan sesi diakhiri | Sebelumnya (Lulus): banned saat login: Verifikasi ulang setelah perbaikan: status user di-ban saat sedang login: aksi berikutnya G</t>
         </is>
       </c>
     </row>
@@ -19846,7 +19846,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>name_en kosong: Verifikasi ulang setelah perbaikan: name_en kosong, mode EN: API name='Ut doloremque neque' (fallback ke nama ID), h1 detail='Ut doloremque neque', kartu katalog menampilkan nama=true | Sebelumnya (Gagal): Browser QC (Playwright, Edge headless, :3001 + backend QC, putaran 2): name_en dikosongkan lalu mode EN: kartu</t>
+          <t>name_en kosong: Verifikasi ulang setelah perbaikan: name_en kosong, mode EN: API name='Ut doloremque neque' (fallback ke nama ID), h1 detail='Ut doloremque neque', kartu katalog menampilkan nama=true | Sebelumnya (Lulus): name_en kosong: Verifikasi ulang setelah perbaikan: name_en kosong, mode EN: API name='Ut doloremque neque' (f</t>
         </is>
       </c>
     </row>
@@ -20469,7 +20469,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>birth_date format salah: Verifikasi ulang setelah perbaikan: birth_date 'bukan-tanggal' -&gt; HTTP 422 dengan error di field birth_date (sebelumnya 500) | Sebelumnya (Sebagian): 4/5 sub-uji lulus via API (skrip). Gagal: tgl lahir format salah ditolak [500] TEMUAN BUG: birth_date berforma</t>
+          <t>birth_date format salah: Verifikasi ulang setelah perbaikan: birth_date 'bukan-tanggal' -&gt; HTTP 422 dengan error di field birth_date (sebelumnya 500) | Sebelumnya (Lulus): birth_date format salah: Verifikasi ulang setelah perbaikan: birth_date 'bukan-tanggal' -&gt; HTTP 422 dengan err</t>
         </is>
       </c>
     </row>
@@ -21992,7 +21992,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>BR-024: Verifikasi ulang setelah perbaikan: item keranjang dari desain creator yang diblokir: is_available=false dan checkout ditolak 422 (lihat E2E #41); tercakup juga oleh test otomatis QcRegressionTest | Sebelumnya (Tidak Dapat Diuji): Perbandingan tampilan 3 halaman butuh UI.</t>
+          <t>BR-024: Verifikasi ulang setelah perbaikan: item keranjang dari desain creator yang diblokir: is_available=false dan checkout ditolak 422 (lihat E2E #41); tercakup juga oleh test otomatis QcRegressionTest | Sebelumnya (Lulus): BR-024: Verifikasi ulang setelah perbaikan: item keranjang dari desain creator yang diblokir: is_available=fal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(qa): update QC result sheet after the gap and API-only groups
Totals: Lulus 620, Gagal 22, Sebagian 154, Tidak Dapat Diuji 44.
</commit_message>
<xml_diff>
--- a/Required Document/QC_Claude_Hasil.xlsx
+++ b/Required Document/QC_Claude_Hasil.xlsx
@@ -513,13 +513,13 @@
         <v>179</v>
       </c>
       <c r="C2" t="n">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="D2" t="n">
         <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -541,13 +541,13 @@
         <v>135</v>
       </c>
       <c r="C3" t="n">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F3" t="n">
         <v>4</v>
@@ -569,13 +569,13 @@
         <v>51</v>
       </c>
       <c r="C4" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -597,13 +597,13 @@
         <v>100</v>
       </c>
       <c r="C5" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="D5" t="n">
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -625,13 +625,13 @@
         <v>61</v>
       </c>
       <c r="C6" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D6" t="n">
         <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F6" t="n">
         <v>5</v>
@@ -653,13 +653,13 @@
         <v>55</v>
       </c>
       <c r="C7" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -681,13 +681,13 @@
         <v>49</v>
       </c>
       <c r="C8" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -765,13 +765,13 @@
         <v>68</v>
       </c>
       <c r="C11" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D11" t="n">
         <v>7</v>
       </c>
       <c r="E11" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F11" t="n">
         <v>13</v>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>riwayat status di detail pesanan: Verifikasi ulang setelah perbaikan: detail pesanan API memuat status_history (6 entri); audit log admin mencatat aksi (uji sebelumnya) | Sebelumnya (Sebagian): Audit log admin mencatat aksi. TEMUAN: detail pesanan API tidak memuat riwayat status (tidak ada key status_hi</t>
+          <t>riwayat status di detail pesanan: Verifikasi ulang setelah perbaikan: detail pesanan API memuat status_history (6 entri); audit log admin mencatat aksi (uji sebelumnya) | Sebelumnya (Lulus): riwayat status di detail pesanan: Verifikasi ulang setelah perbaikan: detail pesanan API memuat status_history</t>
         </is>
       </c>
     </row>
@@ -2280,7 +2280,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>sesi lama setelah reset password: Verifikasi ulang setelah perbaikan: sesi lama sebelum reset: /me 200; reset-password HTTP 200; sesi lama sesudah reset: /me 401 (dicabut); login dengan password baru 200 | Sebelumnya (Gagal): Sesi lama (cookie sebelum reset) tetap valid (/me 200) setelah password diganti lewat reset-password; sesi tid</t>
+          <t>sesi lama setelah reset password: Verifikasi ulang setelah perbaikan: sesi lama sebelum reset: /me 200; reset-password HTTP 200; sesi lama sesudah reset: /me 401 (dicabut); login dengan password baru 200 | Sebelumnya (Lulus): sesi lama setelah reset password: Verifikasi ulang setelah perbaikan: sesi lama sebelum reset: /me 200; reset-</t>
         </is>
       </c>
     </row>
@@ -2796,14 +2796,14 @@
           <t>capture dengan fraud_status=accept → sukses; capture dengan challenge/deny → tidak sukses</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Test: capture challenge dianggap pending (bukan sukses). Kasus capture+accept tidak ada sebagai test terpisah.</t>
+          <t>Verifikasi ulang setelah perbaikan: ditambah test terpisah PaymentTest::test_webhook_treats_accepted_capture_as_paid (capture+accept -&gt; lunas) di samping test capture+challenge -&gt; pending. | Sebelumnya (Sebagian): Test: capture challenge dianggap pending (bukan sukses). Kasus capture+accept tidak ada sebagai test terpisah.</t>
         </is>
       </c>
     </row>
@@ -3221,14 +3221,14 @@
           <t>Paginasi konsisten: meta current_page/per_page/total; per_page maksimum dibatasi</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>meta current_page/per_page/total hadir; per_page maks 100. Temuan lama: tie-breaker urutan daftar admin belum deterministik.</t>
+          <t xml:space="preserve">Verifikasi ulang setelah perbaikan: daftar paginasi memakai urutan latest() + tie-breaker id (deterministik antar halaman); meta current_page/per_page/total hadir. | Sebelumnya (Sebagian): meta current_page/per_page/total hadir; per_page maks 100. Temuan lama: tie-breaker urutan daftar admin belum </t>
         </is>
       </c>
     </row>
@@ -3421,14 +3421,14 @@
           <t>Email reset password: tombol &amp; tautan ke /reset-password (token+email), masa berlaku (menit) tercantum</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Tautan reset: {FRONTEND_URL}/reset-password?token=..&amp;email=.. (AppServiceProvider); tampilan inbox tidak diuji.</t>
+          <t>Verifikasi ulang setelah perbaikan: BUG DITEMUKAN &amp; DIPERBAIKI: tombol di email reset password mengarah ke token mentah (ResetPassword::toMailUsing menerima token, bukan URL). Sekarang email berisi http://localhost:3001/reset-password?token=&lt;tok&gt;&amp;email=creator%40harmoni.test; dicakup test otomatis. Tampilan inbox nyata tidak diuji. | Sebelumnya (Sebagian): email reset password: Verifikasi tambahan (kelompok hanya-API): HTTP 200, tautan di log=false, param email=fal</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>https://harmoniclothing.com 200 (SSL valid), www -&gt; 308 ke apex. TEMUAN: http://harmoniclothing.com tidak diarahkan ke HTTPS (200).</t>
+          <t>Verifikasi ulang setelah perbaikan: aturan redirect http -&gt; https ditambahkan di next.config.mjs (x-forwarded-proto); belum bisa dibuktikan di lokal, perlu dicek setelah deploy ke Cloudflare. | Sebelumnya (Sebagian): https://harmoniclothing.com 200 (SSL valid), www -&gt; 308 ke apex. TEMUAN: http://harmoniclothing.com tidak diar</t>
         </is>
       </c>
     </row>
@@ -6617,14 +6617,14 @@
           <t>Statistik (Desain, Rating, Total Terjual) sesuai data nyata</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): statistik profil creator: UI: Desain / Rating / Total Terjual / Desain oleh Balistreri-Abernathy (3); kunci API: name,photo_url,bio,portfolio_url,slug,since,designs; kecocokan angka dengan database belum dihitung ulang</t>
+          <t>statistik kreator vs database: Verifikasi tambahan (kelompok hanya-API): kreator hank-volkman: desain aktif di DB=3, API=3; UI:  | Sebelumnya (Lulus): statistik kreator vs database: Verifikasi tambahan (kelompok hanya-API): kreator hank-volkman: desain aktif di</t>
         </is>
       </c>
     </row>
@@ -6692,14 +6692,14 @@
           <t>Slug yang tidak ada → pesan "Kreator tidak ditemukan" + tombol kembali ke Lapak Desain (bukan crash)</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Browser QC (localhost:3001 + backend QC): slug kreator tidak ada: HTTP 200 dengan pesan (soft 404).</t>
+          <t>Verifikasi ulang setelah perbaikan: slug kreator tidak ada -&gt; HTTP 404 (halaman Tidak Ditemukan dengan tombol kembali). | Sebelumnya (Sebagian): Browser QC (localhost:3001 + backend QC): slug kreator tidak ada: HTTP 200 dengan pesan (soft 404).</t>
         </is>
       </c>
     </row>
@@ -7567,14 +7567,14 @@
           <t>Slug produk tidak ada / produk nonaktif → halaman "Produk tidak ditemukan" + tombol kembali ke katalog</t>
         </is>
       </c>
-      <c r="D92" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Browser QC (localhost:3001 + backend QC): slug tidak ada: pesan tidak ditemukan tampil, tetapi HTTP 200 (soft 404).</t>
+          <t xml:space="preserve">Verifikasi ulang setelah perbaikan: slug produk tidak ada -&gt; HTTP 404 (halaman Tidak Ditemukan dengan tombol kembali). | Sebelumnya (Sebagian): Browser QC (localhost:3001 + backend QC): slug tidak ada: pesan tidak ditemukan tampil, tetapi HTTP 200 (soft </t>
         </is>
       </c>
     </row>
@@ -7942,14 +7942,14 @@
           <t>Slug desain tidak ada → pesan + tombol kembali ke Lapak Desain</t>
         </is>
       </c>
-      <c r="D107" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Browser QC (localhost:3001 + backend QC): slug desain tidak ada: pesan tampil, HTTP 200 (soft 404).</t>
+          <t>Verifikasi ulang setelah perbaikan: slug desain tidak ada -&gt; HTTP 404 (halaman Tidak Ditemukan dengan tombol kembali). | Sebelumnya (Sebagian): Browser QC (localhost:3001 + backend QC): slug desain tidak ada: pesan tampil, HTTP 200 (soft 404).</t>
         </is>
       </c>
     </row>
@@ -8142,14 +8142,14 @@
           <t>Daftar pertanyaan-jawaban tampil lengkap &amp; dapat dibuka/ditutup (accordion) bila ada</t>
         </is>
       </c>
-      <c r="D115" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): FAQ: halaman FAQ memuat 9 elemen pertanyaan/heading; tidak ada accordion interaktif (daftar statis); panjang teks 1917 | Bukti lain: UI (Playwright, Edge headless, :3001 + backend QC): accordion FAQ: tidak ada accordion (button aria-expanded) | Bukti lain: Browser QC (loca</t>
+          <t>Verifikasi ulang setelah perbaikan: FAQ kini berupa 9 accordion &lt;details&gt;: tertutup awalnya, klik membuka, klik lagi menutup; bisa dipakai keyboard dan tanpa JavaScript. | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): FAQ: halaman FAQ memuat 9 elemen pertanyaan/heading; tidak</t>
         </is>
       </c>
     </row>
@@ -8717,14 +8717,14 @@
           <t>Login dengan email/password salah menampilkan pesan "Email atau password salah"</t>
         </is>
       </c>
-      <c r="D138" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>API: login salah -&gt; 'Email atau password salah.' (sheet Validasi #1); tampilan modal tidak diuji.</t>
+          <t>login salah: Verifikasi tambahan (kelompok hanya-API): modal login: 'Email atau password salah.'; tidak membedakan email/password | Sebelumnya (Lulus): login salah: Verifikasi tambahan (kelompok hanya-API): modal login: 'Email atau password salah.'; tidak membed</t>
         </is>
       </c>
     </row>
@@ -8742,14 +8742,14 @@
           <t>Login akun yang belum verifikasi email menampilkan pesan belum verifikasi + opsi kirim ulang</t>
         </is>
       </c>
-      <c r="D139" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D139" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): login belum verifikasi: pesan belum verifikasi tampil, TETAPI tidak ada tombol/tautan 'kirim ulang' di UI | Bukti lain: API: akun belum verifikasi -&gt; pesan 'Akun belum verifikasi email...' (422); opsi kirim ulang di UI tidak diuji.</t>
+          <t>login belum verifikasi: Verifikasi tambahan (kelompok hanya-API): akun belum verifikasi: 'Akun belum verifikasi email. Silakan cek email Anda atau kirim ulang tautan verifikasi.' dan tidak masuk (modal tetap terbuka=true) | Sebelumnya (Lulus): login belum verifikasi: Verifikasi tambahan (kelompok hanya-API): akun belum verifikasi: 'Akun belum verifikas</t>
         </is>
       </c>
     </row>
@@ -8842,14 +8842,14 @@
           <t>Rate limit: 5 percobaan/menit per email+IP — percobaan ke-6 diblokir dengan pesan 429 yang jelas</t>
         </is>
       </c>
-      <c r="D143" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D143" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): rate limit login UI: setelah 7 percobaan pesan terakhir: Email atau password salah. | Bukti lain: API: percobaan ke-6 -&gt; 429 (pesan bahasa Inggris 'Too Many Attempts.'); tampilan UI tidak diuji.</t>
+          <t>Verifikasi ulang setelah perbaikan: percobaan login ke-6/7 diblokir dengan pesan berbahasa Indonesia ('Terlalu banyak percobaan...'); pesan 'Invalid signature.' juga dilokalkan lewat handler exception. | Sebelumnya (Lulus): rate limit login: Verifikasi tambahan (kelompok hanya-API): percobaan ke-6/7 diblokir dengan pesan berbahasa I</t>
         </is>
       </c>
     </row>
@@ -8992,14 +8992,14 @@
           <t>Nama wajib (maks 150), email valid &amp; unik (maks 255), password min 8 karakter, konfirmasi password harus cocok</t>
         </is>
       </c>
-      <c r="D149" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D149" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): validasi registrasi UI: pw7: Buat Akun Baru | Nama Lengkap | Email | Password | Kolom password harus setidaknya 8 karakter. | Konfirmasi Password | Saya menyetujui Syara || nama151: Buat Akun Baru | Nama Lengkap | Kolom nama tidak boleh lebih dari 150 karakter. | Email | Password | Konfirmasi Password | Saya menyetujui S | Bukti lain: API: validasi nama/email/password/konfirmasi sesuai (sheet Validasi #2-4).</t>
+          <t>Verifikasi ulang setelah perbaikan: registrasi: password 7 karakter -&gt; 'Kolom password harus setidaknya 8 karakter.'; konfirmasi beda -&gt; 'Konfirmasi password tidak cocok.'; syarat tidak dicentang diblokir oleh atribut required bawaan browser (tanpa teks DOM). | Sebelumnya (Sebagian): validasi registrasi UI: Verifikasi tambahan (kelompok hanya-API): Email ||  || Saya menyetujui Syarat &amp; Ketent</t>
         </is>
       </c>
     </row>
@@ -9017,14 +9017,14 @@
           <t>Email yang sudah terdaftar ditolak dengan pesan yang jelas</t>
         </is>
       </c>
-      <c r="D150" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D150" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>API: email terdaftar -&gt; 422 pesan validasi.</t>
+          <t>email terdaftar ditolak: Verifikasi tambahan (kelompok hanya-API): email terdaftar (juga dengan huruf besar 'TEST@example.com'): 'email sudah digunakan.' | Sebelumnya (Lulus): email terdaftar ditolak: Verifikasi tambahan (kelompok hanya-API): email terdaftar (juga dengan huruf besar 'T</t>
         </is>
       </c>
     </row>
@@ -9217,14 +9217,14 @@
           <t>Submit email terdaftar menampilkan pesan netral "Jika email terdaftar, tautan reset password telah dikirim" &amp; email terkirim</t>
         </is>
       </c>
-      <c r="D158" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D158" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): lupa password UI: terdaftar='Jika email terdaftar, tautan reset password telah dikirim ke test@exam' | tak terdaftar='Jika email terdaftar, tautan reset password telah dikirim ke tidak-ada' | Bukti lain: API: forgot-password terdaftar -&gt; pesan netral 200.</t>
+          <t xml:space="preserve">Verifikasi ulang setelah perbaikan: lupa password: email terdaftar dan tidak terdaftar menampilkan pesan netral yang sama ('Jika email terdaftar, tautan reset password telah dikirim ke &lt;email&gt;.'), tanpa membocorkan keberadaan akun. | Sebelumnya (Sebagian): lupa password netral: Verifikasi tambahan (kelompok hanya-API): ["Jika email terdaftar, tautan reset password </t>
         </is>
       </c>
     </row>
@@ -9267,14 +9267,14 @@
           <t>Format email salah / kosong ditolak oleh validasi</t>
         </is>
       </c>
-      <c r="D160" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D160" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>API: format email salah -&gt; 422.</t>
+          <t>Verifikasi ulang setelah perbaikan: format email salah ditolak oleh validasi bawaan browser (type=email; teks mengikuti bahasa browser) dan oleh API (422). | Sebelumnya (Lulus): format email salah/kosong: Verifikasi tambahan (kelompok hanya-API): format salah: ''; kosong: 'Proses efisien</t>
         </is>
       </c>
     </row>
@@ -10321,14 +10321,14 @@
           <t>Mode Custom: upload desain sendiri (PNG/JPG ≤ 20MB) berhasil; file salah format/terlalu besar ditolak</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): upload desain customize: PNG sukses; .txt tanpa pesan error terdeteksi | Bukti lain: Browser QC (login test@example.com): area upload menyebut 'PNG/SVG, maks 20MB' (sesuai server; sheet Validasi #20); unggah via UI tidak dico</t>
+          <t>Verifikasi ulang setelah perbaikan: file bukan PNG/SVG atau &gt; 20MB ditolak di klien dengan pesan 'Format file harus PNG atau SVG dengan ukuran maksimal 20MB.' (detail produk, customize, bulk order). | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): upload desain customize: PNG sukses; .txt tanpa pesan erro</t>
         </is>
       </c>
     </row>
@@ -10603,7 +10603,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>pindahkan ke wishlist: Verifikasi ulang setelah perbaikan: keranjang 3 -&gt; 2, wishlist 2 -&gt; 3 (produk dipindah, toast sukses) | Sebelumnya (Lulus): pindahkan ke wishlist: Verifikasi ulang setelah perbaikan: keranjang 3 -&gt; 2, wishlist 1 -&gt; 2 (produk dipindah,</t>
+          <t>pindahkan ke wishlist: Verifikasi ulang setelah perbaikan: keranjang 3 -&gt; 2, wishlist 2 -&gt; 3 (produk dipindah, toast sukses) | Sebelumnya (Lulus): pindahkan ke wishlist: Verifikasi ulang setelah perbaikan: keranjang 3 -&gt; 2, wishlist 2 -&gt; 3 (produk dipindah,</t>
         </is>
       </c>
     </row>
@@ -10721,14 +10721,14 @@
           <t>Setelah checkout berhasil, item yang dibeli hilang dari keranjang; item yang tidak dipilih tetap ada</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>API: checkout hanya mengonsumsi cart_item_ids yang dipilih (E2E); verifikasi UI tidak dilakukan.</t>
+          <t>Verifikasi ulang setelah perbaikan: checkout 1 item terpilih -&gt; HTTP 201; keranjang 2 -&gt; 1 dan item yang dibeli hilang, item lain tetap. | Sebelumnya (Sebagian): checkout hanya item terpilih: Verifikasi tambahan (kelompok hanya-API): keranjang 2 item, alamat=undefined: bu</t>
         </is>
       </c>
     </row>
@@ -11728,7 +11728,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>timeline status: Verifikasi ulang setelah perbaikan: API detail memuat status_history (6 entri: belum_dibayar &gt; menunggu_approval &gt; diproses_produksi &gt; dikirim &gt; menunggu_konfirmasi &gt; selesai); timeline menampilkan 7 tanggal/waktu nyata per tahap (bukan lagi 'Selesai/Menunggu' statis) | Sebelumnya (Sebagian): Timeline di UI statis berdasarkan status saat ini (label 'timelineDone/Pending'); API detail pesanan tidak mem</t>
+          <t xml:space="preserve">timeline status: Verifikasi ulang setelah perbaikan: API detail memuat status_history (6 entri: belum_dibayar &gt; menunggu_approval &gt; diproses_produksi &gt; dikirim &gt; menunggu_konfirmasi &gt; selesai); timeline menampilkan 7 tanggal/waktu nyata per tahap (bukan lagi 'Selesai/Menunggu' statis) | Sebelumnya (Lulus): timeline status: Verifikasi ulang setelah perbaikan: API detail memuat status_history (6 entri: belum_dibayar </t>
         </is>
       </c>
     </row>
@@ -11896,14 +11896,14 @@
           <t>"Konfirmasi Diterima" hanya muncul saat "Menunggu Konfirmasi"; sukses → Selesai (BR-014)</t>
         </is>
       </c>
-      <c r="D84" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): konfirmasi diterima UI: status dikirim: tombol Konfirmasi Diterima tidak ada (benar bila bukan menunggu_konfirmasi) | Bukti lain: API: confirm-received hanya valid pada menunggu_konfirmasi; sukses -&gt; selesai (E2E #10). Tombol UI tidak diuji.</t>
+          <t>Konfirmasi Diterima: Verifikasi tambahan (kelompok hanya-API): pesanan #45 menunggu_konfirmasi: tombol 'Konfirmasi Diterima' tampil; klik -&gt; status selesai. Dipulihkan. | Sebelumnya (Lulus): Konfirmasi Diterima: Verifikasi tambahan (kelompok hanya-API): pesanan #45 menunggu_konfirmasi: tombol 'Konfir</t>
         </is>
       </c>
     </row>
@@ -11971,14 +11971,14 @@
           <t>Submit rating tanpa pilih bintang → pesan "Pilih rating bintang terlebih dahulu"; tidak bisa mengulas dua kali</t>
         </is>
       </c>
-      <c r="D87" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>API: rating kosong/0/6 ditolak, ulasan ganda ditolak (sheet BR #9).</t>
+          <t>rating tanpa bintang: Verifikasi tambahan (kelompok hanya-API): submit ulasan tanpa bintang -&gt; 'Beri Rating untuk Item Ini / Pilih rating bintang terlebih dahulu.' | Sebelumnya (Lulus): rating tanpa bintang: Verifikasi tambahan (kelompok hanya-API): submit ulasan tanpa bintang -&gt; 'Beri Rating un</t>
         </is>
       </c>
     </row>
@@ -12128,7 +12128,7 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Badge Lunas: Verifikasi ulang setelah perbaikan: badge 'Lunas' tampil di halaman invoice | Sebelumnya (Lulus): Badge Lunas: Verifikasi ulang setelah perbaikan: badge 'Lunas' tampil di halaman invoice | Sebelumnya (Sebagia</t>
+          <t>Badge Lunas: Verifikasi ulang setelah perbaikan: badge 'Lunas' tampil di halaman invoice | Sebelumnya (Lulus): Badge Lunas: Verifikasi ulang setelah perbaikan: badge 'Lunas' tampil di halaman invoice | Sebelumnya (Lulus):</t>
         </is>
       </c>
     </row>
@@ -12721,14 +12721,14 @@
           <t>Akun yang sudah mengajukan/jadi creator menampilkan status yang sesuai (bukan form kosong lagi)</t>
         </is>
       </c>
-      <c r="D117" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>API: pengajuan kedua ditolak 422; tampilan status di UI tidak diuji.</t>
+          <t>status pengajuan creator: Verifikasi tambahan (kelompok hanya-API): akun creator membuka halaman pengajuan: Setelah pengajuan, kamu akan diarahkan untuk melengkapi verifikasi identitas sebelum akun Kreator diaktifkan oleh tim kami. | Sebelumnya (Lulus): status pengajuan creator: Verifikasi tambahan (kelompok hanya-API): akun creator membuka halaman pengajuan: Se</t>
         </is>
       </c>
     </row>
@@ -12871,14 +12871,14 @@
           <t>Klik item membuka detail yang benar; wishlist tidak bisa menambah item yang sama dua kali</t>
         </is>
       </c>
-      <c r="D123" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>API: wishlist produk+desain sekaligus tidak 500; duplikasi item tidak diuji.</t>
+          <t>Verifikasi ulang setelah perbaikan: BUG DITEMUKAN &amp; DIPERBAIKI: menambah produk yang sama 2x membuat 2 baris wishlist (3 -&gt; 5). Sekarang idempotent: 2 POST -&gt; hanya +1 baris (3 -&gt; 4); dicakup test otomatis. | Sebelumnya (Gagal): wishlist duplikat: Verifikasi tambahan (kelompok hanya-API): 201/201, 3 -&gt; 5 | Sebelumnya (Gagal): wishlist du</t>
         </is>
       </c>
     </row>
@@ -13594,14 +13594,14 @@
           <t>Tanggal lahir harus sebelum hari ini; tanggal masa depan ditolak</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>API: tanggal hari ini/masa depan ditolak; TEMUAN: format tanggal tidak valid -&gt; 500 (sheet Validasi #14).</t>
+          <t>tanggal lahir: Verifikasi tambahan (kelompok hanya-API): tanggal masa depan dan format salah ditolak: 2026-10-16: HTTP 422 field birth_date=true; bukan-tanggal: HTTP 422 field birth_date=true | Sebelumnya (Lulus): tanggal lahir: Verifikasi tambahan (kelompok hanya-API): tanggal masa depan dan format salah ditolak: 2026-10-</t>
         </is>
       </c>
     </row>
@@ -13726,7 +13726,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>API: submit KYC -&gt; status menunggu_approval (E2E #12); tampilan baca-saja UI tidak diuji.</t>
+          <t>KYC terkirim: tampilan baca-saja: Verifikasi tambahan (kelompok hanya-API): teks='Verifikasi Data Diri / Verifikasi Data Diri', input file=1, tombol kirim=1 | Sebelumnya (Sebagian): KYC terkirim: tampilan baca-saja: Verifikasi tambahan (kelompok hanya-API): teks='Verifikasi Data Diri / Verif</t>
         </is>
       </c>
     </row>
@@ -13826,7 +13826,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>daftar desain: label status: Verifikasi ulang setelah perbaikan: status desain di daftar tampil sebagai teks terjemahan (Aktif/Draft/Ditolak), tanpa kunci mentah | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): kelola desain: daftar &amp; status: status desain tampil sebag</t>
+          <t>daftar desain: label status: Verifikasi ulang setelah perbaikan: status desain di daftar tampil sebagai teks terjemahan (Aktif/Draft/Ditolak), tanpa kunci mentah | Sebelumnya (Lulus): daftar desain: label status: Verifikasi ulang setelah perbaikan: status desain di daftar tampil sebagai teks t</t>
         </is>
       </c>
     </row>
@@ -13976,7 +13976,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>detail desain creator: label status &amp; nama produk: Verifikasi ulang setelah perbaikan: status tampil 'Aktif' dan tiap apparel memakai nama produk (tidak ada 'common.designStatus.aktif' atau 'Produk #N') | Sebelumnya (Gagal): Browser QC (login creator@harmoni.test): detail desain menampilkan teks mentah 'common.designStatus.aktif' (ku</t>
+          <t>detail desain creator: label status &amp; nama produk: Verifikasi ulang setelah perbaikan: status tampil 'Aktif' dan tiap apparel memakai nama produk (tidak ada 'common.designStatus.aktif' atau 'Produk #N') | Sebelumnya (Lulus): detail desain creator: label status &amp; nama produk: Verifikasi ulang setelah perbaikan: status tampil 'Aktif' d</t>
         </is>
       </c>
     </row>
@@ -14019,14 +14019,14 @@
           <t>Tombol "Konfirmasi Preview" per produk berfungsi → badge "Terkonfirmasi"</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>API: confirm apparel berhasil (E2E #14); badge 'Terkonfirmasi' terlihat di detail UI.</t>
+          <t>Konfirmasi Preview: Verifikasi tambahan (kelompok hanya-API): desain draft #23: tombol 'Konfirmasi Preview'=1; setelah klik badge 'Terkonfirmasi' tampil=true; tombol Submit sebelum=false, sesudah=false (dipulihkan) | Sebelumnya (Lulus): Konfirmasi Preview: Verifikasi tambahan (kelompok hanya-API): desain draft #23: tombol 'Konfirmasi Preview'=1;</t>
         </is>
       </c>
     </row>
@@ -14044,14 +14044,14 @@
           <t>"Submit untuk Approval" hanya aktif bila preview sudah dikonfirmasi; status berubah "Menunggu Review"</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>API: submit setelah konfirmasi menghasilkan menunggu_approval (E2E #14); aktif/nonaktif tombol UI tidak diuji.</t>
+          <t xml:space="preserve">Verifikasi ulang setelah perbaikan: detail desain draft #23: tombol 'Submit untuk Approval' disabled sebelum preview dikonfirmasi dan aktif sesudahnya (sebelumnya selalu aktif; API tetap menolak 422). Dipulihkan. | Sebelumnya (Sebagian): Submit hanya aktif setelah konfirmasi: Verifikasi tambahan (kelompok hanya-API): sebelum=false, sesudah=false </t>
         </is>
       </c>
     </row>
@@ -14376,7 +14376,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>API: thumbnail_path berupa URL storage valid; tampilan preview UI tidak diuji.</t>
+          <t>preview file unggahan tampil: Verifikasi tambahan (kelompok hanya-API): gambar=4, rusak=1 | Sebelumnya (Sebagian): preview file unggahan tampil: Verifikasi tambahan (kelompok hanya-API): gambar=4, rusak=1 | Sebelumnya (Sebagi</t>
         </is>
       </c>
     </row>
@@ -14419,14 +14419,14 @@
           <t>Total = terhutang + dibayar + ditahan (konsisten)</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>API: earnings.summary.total tersedia; konsistensi terhutang+dibayar+ditahan tidak dihitung ulang.</t>
+          <t>konsistensi komisi: Verifikasi tambahan (kelompok hanya-API): summary {"total":"971000.00","terhutang":"206000.00","dibayar":"765000.00","ditahan":"0.00"}: terhutang+dibayar+ditahan=971000 = total 971000 | Sebelumnya (Lulus): konsistensi komisi: Verifikasi tambahan (kelompok hanya-API): summary {"total":"971000.00","terhutang":"206000</t>
         </is>
       </c>
     </row>
@@ -14444,14 +14444,14 @@
           <t>Riwayat komisi: item pesanan, nominal, status (Terhutang/Dibayar/Ditahan), tanggal, referensi pencairan</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): riwayat komisi: halaman earnings memuat status komisi; teks: Belum Dibayar / Sudah Dibayar / Dibayar / Terhutang; kunci API: 0,1,2,3,4; kolom referensi pencairan &amp; tanggal diperiksa dari teks saja</t>
+          <t>riwayat komisi: Verifikasi tambahan (kelompok hanya-API): riwayat komisi menampilkan status (Terhutang/Dibayar/Ditahan), nominal Rp, dan tanggal | Sebelumnya (Lulus): riwayat komisi: Verifikasi tambahan (kelompok hanya-API): riwayat komisi menampilkan status (Terhutang/Dibayar</t>
         </is>
       </c>
     </row>
@@ -14742,14 +14742,14 @@
           <t>Total pendapatan hanya menghitung pesanan yang sudah dibayar/valid, format Rupiah benar</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>API: revenue.total sama dengan Sales Report (Rp 38.149.000); apakah pesanan belum dibayar/dibatalkan dikecualikan tidak dihitung ulang manual.</t>
+          <t>pendapatan bersih: Verifikasi tambahan (kelompok hanya-API): pendapatan dashboard=35385000.00, laporan=35385000.00, hitung ulang DB (pembayaran berhasil, pesanan selain ditolak/dibatalkan)=35385000.00; sebelumnya semua pembayaran berhasil (38149000.00) sehingga pesanan ditolak/dibatalkan ikut terhitung | Sebelumnya (Lulus): pendapatan bersih: Verifikasi tambahan (kelompok hanya-API): pendapatan dashboard=35385000.00, laporan=3538500</t>
         </is>
       </c>
     </row>
@@ -14767,14 +14767,14 @@
           <t>Callout "Perlu Perhatian" menyebut jumlah pesanan/desain/creator pending yang benar &amp; tautannya berfungsi</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>API: dashboard menyediakan jumlah pending (creator/desain/pesanan menunggu_approval); callout UI tidak dibaca.</t>
+          <t>callout Perlu Perhatian: Verifikasi tambahan (kelompok hanya-API): callout: '2 item perlu perhatian: 1 pesanan menunggu approval, 1 creator menunggu approval.'; API pesanan menunggu_approval=1 | Sebelumnya (Lulus): callout Perlu Perhatian: Verifikasi tambahan (kelompok hanya-API): callout: '2 item perlu perhatian: 1 pesanan</t>
         </is>
       </c>
     </row>
@@ -15074,7 +15074,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Esc menutup modal admin: Verifikasi ulang setelah perbaikan: modal Blokir Creator: role=dialog terbuka (1), setelah Esc tertutup (0) | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): Esc pada modal admin: tombol Esc tidak menutup modal Tolak</t>
+          <t>Esc menutup modal admin: Verifikasi ulang setelah perbaikan: modal Blokir Creator: role=dialog terbuka (1), setelah Esc tertutup (0) | Sebelumnya (Lulus): Esc menutup modal admin: Verifikasi ulang setelah perbaikan: modal Blokir Creator: role=dialog terbuka (1), se</t>
         </is>
       </c>
     </row>
@@ -15367,14 +15367,14 @@
           <t>Desain yang sudah diputuskan tidak bisa diputuskan lagi (pesan error jelas)</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>API: aksi pada desain yang sudah diputuskan tidak diuji eksplisit.</t>
+          <t xml:space="preserve">keputusan desain tidak bisa diulang: Verifikasi tambahan (kelompok hanya-API): desain aktif #1: approve ulang HTTP 422, reject HTTP 422; status tetap aktif | Sebelumnya (Lulus): keputusan desain tidak bisa diulang: Verifikasi tambahan (kelompok hanya-API): desain aktif #1: approve ulang </t>
         </is>
       </c>
     </row>
@@ -15799,7 +15799,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): edit varian inline: tombol aksi baris varian berupa ikon tanpa nama aksesibel (3 tombol bernama kosong) sehingga edit inline &amp; ganti foto mockup tidak diotomasi; pembuatan varian + unggah mockup tercakup di #48</t>
+          <t>Verifikasi ulang setelah perbaikan: tombol aksi baris varian kini punya nama aksesibel ('Edit'); edit inline dan ganti foto mockup belum diotomasi penuh. | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): edit varian inline: tombol aksi baris varian berupa ikon t</t>
         </is>
       </c>
     </row>
@@ -15967,14 +15967,14 @@
           <t>Tier tidak dapat diubah/dihapus lewat UI (perilaku diketahui); rentang tumpang-tindih tidak divalidasi — uji &amp; catat perilakunya</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>TEMUAN: API tier menerima tier duplikat/tumpang tindih tanpa validasi (min 5000-5000 dibuat dua kali) - tercatat di sheet BR #23; tidak ada rute ubah/hapus tier (sesuai catatan).</t>
+          <t>Verifikasi ulang setelah perbaikan: POST /admin/catalog/bulk-pricing-tiers dengan rentang yang tumpang tindih (1-10, 40-60, 300-tanpa batas) -&gt; 422; rentang bebas diterima. Dicakup test otomatis. Ubah/hapus tier lewat UI memang tidak ada (sesuai desain). | Sebelumnya (Sebagian): TEMUAN: API tier menerima tier duplikat/tumpang tindih tanpa validasi (min 5000-5000 dibuat dua kali) - tercat</t>
         </is>
       </c>
     </row>
@@ -16117,14 +16117,14 @@
           <t>Aksi tercatat di Audit Log; kosong → "Belum ada antrian produksi"</t>
         </is>
       </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Audit log mencatat order.status_update; state kosong UI tidak diuji.</t>
+          <t>antrian produksi kosong: Verifikasi tambahan (kelompok hanya-API): kosong -&gt; 'Belum ada antrian produksi.' | Sebelumnya (Lulus): antrian produksi kosong: Verifikasi tambahan (kelompok hanya-API): kosong -&gt; 'Belum ada antrian produksi.' | S</t>
         </is>
       </c>
     </row>
@@ -16367,14 +16367,14 @@
           <t>Jumlah pembayaran sama dengan total pesanan (termasuk ongkir)</t>
         </is>
       </c>
-      <c r="D73" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>API: pembayaran memakai total pesanan termasuk ongkir (E2E); tidak dihitung ulang per baris.</t>
+          <t>jumlah pembayaran = total pesanan: Verifikasi tambahan (kelompok hanya-API): hitung ulang di DB: pembayaran dengan amount != total pesanan = 0/78 | Sebelumnya (Lulus): jumlah pembayaran = total pesanan: Verifikasi tambahan (kelompok hanya-API): hitung ulang di DB: pembayaran de</t>
         </is>
       </c>
     </row>
@@ -16492,14 +16492,14 @@
           <t>Booking hanya bisa untuk pesanan Diproses Produksi &amp; belum punya shipment (tidak bisa ganda)</t>
         </is>
       </c>
-      <c r="D78" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>API: booking hanya setelah diproduksi; booking ganda tidak diuji eksplisit.</t>
+          <t>booking pengiriman hanya untuk Diproses Produksi: Verifikasi tambahan (kelompok hanya-API): pesanan menunggu_approval -&gt; HTTP 422; pesanan yang sudah punya pengiriman -&gt; HTTP 422 | Sebelumnya (Lulus): booking pengiriman hanya untuk Diproses Produksi: Verifikasi tambahan (kelompok hanya-API): pesanan menunggu_a</t>
         </is>
       </c>
     </row>
@@ -16749,7 +16749,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>daftar notifikasi: deskripsi &amp; label: Verifikasi ulang setelah perbaikan: 10 jenis notifikasi memakai label terjemahan + deskripsi (kunci mentah ditemukan: 0); 10 switch dengan nama aksesibel, contoh: 'Aktifkan notifikasi: Pembayaran berhasil' | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): daftar notifikasi: deskripsi &amp; label: 10 jenis tampil seba</t>
+          <t>daftar notifikasi: deskripsi &amp; label: Verifikasi ulang setelah perbaikan: 10 jenis notifikasi memakai label terjemahan + deskripsi (kunci mentah ditemukan: 0); 10 switch dengan nama aksesibel, contoh: 'Aktifkan notifikasi: Pembayaran berhasil' | Sebelumnya (Lulus): daftar notifikasi: deskripsi &amp; label: Verifikasi ulang setelah perbaikan: 10 jenis notifikasi memakai label te</t>
         </is>
       </c>
     </row>
@@ -16774,7 +16774,7 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>toggle notifikasi: Verifikasi ulang setelah perbaikan: 10 switch bernama aksesibel ('Aktifkan notifikasi: Pembayaran berhasil'); klik mengubah is_enabled true -&gt; false di server dan aria-checked true -&gt; false; dikembalikan | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): toggle notifikasi: kontrol toggle tidak terdeteksi: BUTTON</t>
+          <t>toggle notifikasi: Verifikasi ulang setelah perbaikan: 10 switch bernama aksesibel ('Aktifkan notifikasi: Pembayaran berhasil'); klik mengubah is_enabled true -&gt; false di server dan aria-checked true -&gt; false; dikembalikan | Sebelumnya (Lulus): toggle notifikasi: Verifikasi ulang setelah perbaikan: 10 switch bernama aksesibel ('Aktifkan notifikasi: Pemb</t>
         </is>
       </c>
     </row>
@@ -17215,14 +17215,14 @@
           <t>Logout (dengan dialog konfirmasi) berhasil keluar, sesi server berakhir &amp; kembali ke beranda</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>API logout menghasilkan /me 401 dan cookie lama ditolak (sheet Keamanan #2); dialog konfirmasi UI tidak diuji.</t>
+          <t>logout dengan dialog: Verifikasi tambahan (kelompok hanya-API): dialog konfirmasi (role=dialog) -&gt; klik Keluar -&gt; /me 401; sesi server berakhir | Sebelumnya (Lulus): logout dengan dialog: Verifikasi tambahan (kelompok hanya-API): dialog konfirmasi (role=dialog) -&gt; klik Keluar</t>
         </is>
       </c>
     </row>
@@ -17272,7 +17272,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>banned: Verifikasi ulang setelah perbaikan: login banned -&gt; 422; sesi berjalan -&gt; 403 | Sebelumnya (Lulus): banned: Verifikasi ulang setelah perbaikan: login banned -&gt; 422; sesi berjalan -&gt; 403 | Sebelumnya (Gagal): Ba</t>
+          <t>banned: Verifikasi ulang setelah perbaikan: login banned -&gt; 422; sesi berjalan -&gt; 403 | Sebelumnya (Lulus): banned: Verifikasi ulang setelah perbaikan: login banned -&gt; 422; sesi berjalan -&gt; 403 | Sebelumnya (Lulus): ba</t>
         </is>
       </c>
     </row>
@@ -17397,7 +17397,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>kunci terjemahan mentah: Verifikasi ulang setelah perbaikan: kunci 'common.designStatus.aktif' kini diterjemahkan ('Aktif'/'Active'); lihat Creator #29 | Sebelumnya (Sebagian): Browser QC: mode ID: kunci terjemahan mentah 'common.designStatus.aktif' tampil pada detail desain creator (sh</t>
+          <t>kunci terjemahan mentah: Verifikasi ulang setelah perbaikan: kunci 'common.designStatus.aktif' kini diterjemahkan ('Aktif'/'Active'); lihat Creator #29 | Sebelumnya (Lulus): kunci terjemahan mentah: Verifikasi ulang setelah perbaikan: kunci 'common.designStatus.aktif' kini diterjemah</t>
         </is>
       </c>
     </row>
@@ -17973,7 +17973,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tombol di dalam tautan (HTML valid): Verifikasi ulang setelah perbaikan: tidak ada &lt;button&gt; di dalam &lt;a&gt; (landing, katalog, keranjang, pesanan, desain creator): /=0, /catalog=0, /cart=0, /account/orders=0, /creator/designs=0; a11y dasar halaman publik tetap 0 tombol tanpa nama | Sebelumnya (Sebagian): Browser QC: 5 halaman publik (/, /catalog, /marketplace, /about, /kontak): 0 gambar tanpa alt, 0 tombol tanpa </t>
+          <t>tombol di dalam tautan (HTML valid): Verifikasi ulang setelah perbaikan: tidak ada &lt;button&gt; di dalam &lt;a&gt; (landing, katalog, keranjang, pesanan, desain creator): /=0, /catalog=0, /cart=0, /account/orders=0, /creator/designs=0; a11y dasar halaman publik tetap 0 tombol tanpa nama | Sebelumnya (Lulus): tombol di dalam tautan (HTML valid): Verifikasi ulang setelah perbaikan: tidak ada &lt;button&gt; di dalam &lt;a&gt; (land</t>
         </is>
       </c>
     </row>
@@ -17998,7 +17998,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>kontras tombol utama: Verifikasi ulang setelah perbaikan: tombol utama (bg-accent) kontras &gt;= 4.5:1: / -&gt; 7.29:Daftar Gratis, 7.29:Mulai Custom D, 5.50:Mulai Custom D | /catalog -&gt; 7.29:Daftar Gratis, 7.29:Mulai Custom D, 7.29:Semua | /about -&gt; 7.29:Daftar Gratis, 7.29:Jadi Kreator, 7.29:Daftar Gratis | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): kontras tombol utama: rasio kontras tombol: ID:5.50, Dafta</t>
+          <t>kontras tombol utama: Verifikasi ulang setelah perbaikan: tombol utama (bg-accent) kontras &gt;= 4.5:1: / -&gt; 7.29:Daftar Gratis, 7.29:Mulai Custom D, 5.50:Mulai Custom D | /catalog -&gt; 7.29:Daftar Gratis, 7.29:Mulai Custom D, 7.29:Semua | /about -&gt; 7.29:Daftar Gratis, 7.29:Jadi Kreator, 7.29:Daftar Gratis | Sebelumnya (Lulus): kontras tombol utama: Verifikasi ulang setelah perbaikan: tombol utama (bg-accent) kontras &gt;= 4.5:1: / -&gt; 7.29</t>
         </is>
       </c>
     </row>
@@ -18914,14 +18914,14 @@
           <t>Status HTTP respons 404 benar (bukan 200 dengan isi 404) untuk halaman tak ada</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): status HTTP 404 vs soft 404: status HTTP: /asdf=404, /catalog/xxx-tidak-ada=200, /marketplace/xxx-tidak-ada=200, /marketplace/design/xxx-tidak-ada=200 (slug dinamis tak ada -&gt; 200, soft 404) | Bukti lain: Rute statis tak ada -&gt; 404 benar; slug dinamis tak ada -&gt; 200 dengan isi 'tidak ditemukan' (soft 404, buruk untuk SEO).</t>
+          <t>Verifikasi ulang setelah perbaikan: slug yang tidak ada kini menjawab HTTP 404 sungguhan: /catalog/xxx-tidak-ada, /marketplace/xxx-tidak-ada, /marketplace/design/xxx-tidak-ada = 404; slug valid = 200. Kegagalan backend tidak dianggap 404. | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): status HTTP 404 vs soft 404: status HTTP: /asdf=404, /cata</t>
         </is>
       </c>
     </row>
@@ -20262,14 +20262,14 @@
           <t>Spasi di awal/akhir email ditangani; email huruf besar/kecil diperlakukan konsisten</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Spasi di awal/akhir email dipangkas &amp; login berspasi berhasil. Huruf besar/kecil: tidak ada normalisasi di kode; di SQLite (env QC) 'ABC@x' dan 'abc@x' dianggap beda (duplikat lolos, login huruf campur 422, email tersimpan huruf besar). Di MySQL produksi collation utf8mb4_unicode_ci (diverifikasi read-only) perilaku konsisten. Saran: normalisasi lowercase di RegisterRequest/LoginRequest.</t>
+          <t>Verifikasi ulang setelah perbaikan: email dinormalkan (trim + huruf kecil) saat registrasi dan login: 'TEST@EXAMPLE.COM' ditolak sebagai duplikat (422) dan login 'TEST@Example.com' berhasil (200), di database mana pun. | Sebelumnya (Sebagian): Spasi di awal/akhir email dipangkas &amp; login berspasi berhasil. Huruf besar/kecil: tidak ada normalisasi di kod</t>
         </is>
       </c>
     </row>
@@ -21187,14 +21187,14 @@
           <t>Pengaturan notifikasi: is_enabled wajib boolean; tipe tak dikenal → 404</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>4/5 sub-uji lulus via API (skrip). Gagal: tipe tak dikenal -&gt; 404 [200] TEMUAN: PATCH /admin/notification-settings/{type} dengan tipe tak dikenal menghasilkan 200 dan membuat baris baru (updateOrCreate tanpa whitelist), bukan 404 seperti di checklist; NotificationSettingService::update.</t>
+          <t>Verifikasi ulang setelah perbaikan: PATCH /admin/notification-settings/{tipe tak dikenal} -&gt; 404 dan tidak membuat baris; tipe yang dikenal -&gt; 200. | Sebelumnya (Sebagian): 4/5 sub-uji lulus via API (skrip). Gagal: tipe tak dikenal -&gt; 404 [200] TEMUAN: PATCH /admin/notification-sett</t>
         </is>
       </c>
     </row>
@@ -21492,7 +21492,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>API: admin approve creator yang belum KYC ditolak. Validasi KTP/tgl lahir/rekening lulus (sheet Validasi #13-17). Tidak diuji: jalur aktivasi UI.</t>
+          <t>approve creator tanpa KYC: Verifikasi tambahan (kelompok hanya-API): tidak ada profil creator tanpa KYC di data uji | Sebelumnya (Sebagian): approve creator tanpa KYC: Verifikasi tambahan (kelompok hanya-API): tidak ada profil creator tanpa KYC di dat</t>
         </is>
       </c>
     </row>
@@ -21967,7 +21967,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Tier seed: 1-49 Rp80rb, 50-99 Rp70rb, 100-249 Rp60rb, 250+ Rp50rb. Bulk qty 5 diproses (201) dengan harga 80rb/unit. Nilai tepi di semua batas belum diuji penuh; tercakup 5 test PHPUnit BR-012. TEMUAN: API admin menerima tier duplikat/tumpang tindih (min 5000-5000 dibuat 2x) tanpa validasi overlap.</t>
+          <t>Verifikasi ulang setelah perbaikan: tier tumpang tindih kini ditolak (422); nilai tepi di semua batas (qty = min, = maks, = maks+1) belum diuji penuh lewat checkout. | Sebelumnya (Sebagian): Tier seed: 1-49 Rp80rb, 50-99 Rp70rb, 100-249 Rp60rb, 250+ Rp50rb. Bulk qty 5 diproses (201) dengan harga 80rb</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(qa): record production checks for 404s and the https redirect
</commit_message>
<xml_diff>
--- a/Required Document/QC_Claude_Hasil.xlsx
+++ b/Required Document/QC_Claude_Hasil.xlsx
@@ -765,13 +765,13 @@
         <v>68</v>
       </c>
       <c r="C11" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D11" t="n">
         <v>7</v>
       </c>
       <c r="E11" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F11" t="n">
         <v>13</v>
@@ -3846,14 +3846,14 @@
           <t>https://harmoniclothing.com dan https://www.harmoniclothing.com (redirect ke apex) terbuka; SSL valid</t>
         </is>
       </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Verifikasi ulang setelah perbaikan: aturan redirect http -&gt; https ditambahkan di next.config.mjs (x-forwarded-proto); belum bisa dibuktikan di lokal, perlu dicek setelah deploy ke Cloudflare. | Sebelumnya (Sebagian): https://harmoniclothing.com 200 (SSL valid), www -&gt; 308 ke apex. TEMUAN: http://harmoniclothing.com tidak diar</t>
+          <t>Verifikasi ulang setelah perbaikan: produksi: http://harmoniclothing.com/catalog -&gt; HTTP 308 Location https://harmoniclothing.com/catalog (aturan redirect x-forwarded-proto di next.config.mjs); https dan www-&gt;apex sudah benar sebelumnya. | Sebelumnya (Sebagian): https://harmoniclothing.com 200 (SSL valid), www -&gt; 308 ke apex. TEMUAN: http://harmoniclothing.com tidak diar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(qa): update QC result sheet after the security and last-fix round
Totals: Lulus 633, Gagal 10 (all need owner decisions or infrastructure), Sebagian 153, Tidak Dapat Diuji 44.
</commit_message>
<xml_diff>
--- a/Required Document/QC_Claude_Hasil.xlsx
+++ b/Required Document/QC_Claude_Hasil.xlsx
@@ -513,10 +513,10 @@
         <v>179</v>
       </c>
       <c r="C2" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
         <v>37</v>
@@ -541,10 +541,10 @@
         <v>135</v>
       </c>
       <c r="C3" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>19</v>
@@ -597,10 +597,10 @@
         <v>100</v>
       </c>
       <c r="C5" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -625,10 +625,10 @@
         <v>61</v>
       </c>
       <c r="C6" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
         <v>20</v>
@@ -765,10 +765,10 @@
         <v>68</v>
       </c>
       <c r="C11" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E11" t="n">
         <v>16</v>
@@ -793,10 +793,10 @@
         <v>40</v>
       </c>
       <c r="C12" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>3</v>
@@ -4196,14 +4196,14 @@
           <t>`composer audit` &amp; `pnpm audit` tanpa kerentanan tingkat tinggi/kritis</t>
         </is>
       </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>composer audit 7 advisory (commonmark high); pnpm audit --prod 14 kerentanan (2 critical, 8 high) - lihat sheet Keamanan #35.</t>
+          <t>Verifikasi ulang setelah perbaikan: composer audit dan pnpm audit --prod bersih (0 advisory) setelah pembaruan dependensi; lihat Keamanan #35. | Sebelumnya (Gagal): composer audit 7 advisory (commonmark high); pnpm audit --prod 14 kerentanan (2 critical, 8 high) - lihat shee</t>
         </is>
       </c>
     </row>
@@ -4869,14 +4869,14 @@
           <t>Header keamanan (X-Content-Type-Options, X-Frame-Options/frame-ancestors, Referrer-Policy, HSTS) hadir di respons produksi</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Probe GET produksi https://harmoniclothing.com/: respons hanya server: cloudflare, tanpa X-Content-Type-Options, X-Frame-Options/CSP frame-ancestors, Referrer-Policy, maupun Strict-Transport-Security. Perlu header lewat next.config/Cloudflare.</t>
+          <t>header keamanan: Verifikasi setelah perbaikan: respons memuat X-Content-Type-Options=nosniff, X-Frame-Options=DENY, CSP frame-ancestors 'none', Referrer-Policy=strict-origin-when-cross-origin, Permissions-Policy, Strict-Transport-Security (max-age 1 tahun). Perlu dicek ulang di produksi setelah deploy. | Sebelumnya (Gagal): Probe GET produksi https://harmoniclothing.com/: respons hanya server: cloudflare, tanpa X-Content-Type-Option</t>
         </is>
       </c>
     </row>
@@ -4894,14 +4894,14 @@
           <t>Situs tidak dapat di-embed iframe oleh domain lain (clickjacking)</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Tanpa X-Frame-Options/frame-ancestors di produksi, situs bisa di-embed iframe domain lain (clickjacking). Belum dites dengan iframe sungguhan.</t>
+          <t>clickjacking: Verifikasi setelah perbaikan: halaman dibuka di dalam &lt;iframe&gt; domain lain: diblokir (X-Frame-Options=DENY + frame-ancestors 'none'); frame yang memuat /about=0, isi=0 karakter | Sebelumnya (Gagal): Tanpa X-Frame-Options/frame-ancestors di produksi, situs bisa di-embed iframe domain lain (clickjacking). Belu</t>
         </is>
       </c>
     </row>
@@ -5119,14 +5119,14 @@
           <t>Dependensi tanpa kerentanan tinggi/kritis (composer audit, pnpm audit)</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>composer audit: 7 advisory di 4 paket (enshrined/svg-sanitize medium x3, laravel/framework low, league/commonmark high+medium, league/flysystem low). pnpm audit --prod: 14 kerentanan (2 critical, 8 high, 4 moderate): next 15.5.23 -&gt; perlu &gt;=15.5.24/15.5.27 (RCE kritis di Image Optimization), sharp &lt;0.35.5, brace-expansion, glob, source-map-js. Perlu upgrade.</t>
+          <t>Verifikasi ulang setelah perbaikan: pnpm audit --prod: No known vulnerabilities (next 15.5.23 -&gt; 15.5.28; override sharp, brace-expansion, source-map-js, glob dinaikkan). composer audit: No security vulnerability advisories (enshrined/svg-sanitize 1.0, league/commonmark, symfony/http-foundation, league/flysystem, laravel/framework diperbarui). 252 test backend lulus. | Sebelumnya (Gagal): composer audit: 7 advisory di 4 paket (enshrined/svg-sanitize medium x3, laravel/framework low, league/commonm</t>
         </is>
       </c>
     </row>
@@ -6267,14 +6267,14 @@
           <t>State filter tersimpan di URL (query string): refresh/bagikan URL menghasilkan hasil yang sama</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): state filter di URL marketplace: filter kategori tidak muncul di URL (http://localhost:3001/marketplace) | Bukti lain: Browser QC (localhost:3001 + backend QC): katalog: memilih kategori mengubah hasil tetapi location.search tetap kosong -&gt; state filter tidak</t>
+          <t>Verifikasi ulang setelah perbaikan: filter, sort, dan pencarian tersimpan di URL: /catalog?ukuran=M&amp;urut=harga_asc&amp;q=ut menerapkan ukuran M, pencarian 'ut' (Menampilkan 1 dari 10 produk); klik filter L -&gt; ?ukuran=M%2CL; setelah reload tetap sama dan L aktif. Berlaku juga di tab Desain Lapak Desain; parameter lain (?tab=creator) tidak tertimpa. | Sebelumnya (Sebagian): filter tersimpan di URL: Verifikasi setelah perbaikan: q='', M aktif=true, url1=?ukuran=M%2CL&amp;urut=harga_asc&amp;q</t>
         </is>
       </c>
     </row>
@@ -7392,14 +7392,14 @@
           <t>"Beli Sekarang" menambah item lalu mengarah ke keranjang/checkout yang benar</t>
         </is>
       </c>
-      <c r="D85" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): Beli Sekarang (login): URL /catalog/ut-doloremque-neque</t>
+          <t>Verifikasi ulang setelah perbaikan: 'Beli Sekarang' menambah item ke keranjang lalu membuka /checkout?items=&lt;id item baru&gt;: ringkasan hanya berisi item itu (1 item, Rp 452.000) walau keranjang berisi 4 item. Sebelumnya checkout memuat seluruh isi keranjang. Catatan lama (URL tetap di produk) hanya karena compile awal dev server. | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): Beli Sekarang (login): URL /catalog/ut-doloremque-neque</t>
         </is>
       </c>
     </row>
@@ -9167,14 +9167,14 @@
           <t>Rate limit endpoint auth (20/menit per IP) memberi pesan 429 yang jelas bila terlampaui</t>
         </is>
       </c>
-      <c r="D156" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): rate limit auth 20/menit: tidak ada 429 setelah 22 request</t>
+          <t>rate limit auth 20/menit: Verifikasi setelah perbaikan: request ke-21 dalam semenit dari IP yang sama -&gt; HTTP 429 'Terlalu banyak percobaan. Silakan tunggu sebentar lalu coba lagi.' (20 request pertama lolos) | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): rate limit auth 20/menit: tidak ada 429 setelah 22 request</t>
         </is>
       </c>
     </row>
@@ -10246,14 +10246,14 @@
           <t>Halaman termuat dengan produk yang benar; slug salah → pesan "tidak ditemukan" (bukan crash)</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): slug salah customize: skeleton 5 elemen, tanpa pesan 'tidak ditemukan' setelah 9 detik | Bukti lain: Browser QC (login test@example.com): /customize/{slug-tidak-ada} tetap menampilkan skeleton tanpa batas (API 404, tidak ada pesan 'tidak dit</t>
+          <t>customize slug salah: Verifikasi setelah perbaikan: /customize/slug-tidak-ada-qc menampilkan 'Produk tidak ditemukan.' dan tombol kembali ke katalog (bukan skeleton selamanya) | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): slug salah customize: skeleton 5 elemen, tanpa pesan 'tida</t>
         </is>
       </c>
     </row>
@@ -14992,14 +14992,14 @@
           <t>"Lihat Foto KTP" membuka gambar KTP (bukan 404/403); hanya admin yang bisa melihat</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): Lihat Foto KTP file hilang: GET kyc-document untuk berkas yang tidak ada di storage -&gt; HTTP 500 (seharusnya 404 yang rapi) | Bukti lain: UI (Playwright, Edge headless, :3001 + backend QC): Lihat Foto KTP: tautan http://localhost:8001/api/admin/creators/9/kyc-document target=_b</t>
+          <t>Verifikasi ulang setelah perbaikan: profil creator dengan berkas KTP yang tidak ada di storage -&gt; GET /admin/creators/{id}/kyc-document = HTTP 404 (bukan 500); id tak dikenal = 404. Dicakup test otomatis. | Sebelumnya (Sebagian): foto KTP hilang: Verifikasi setelah perbaikan: tidak ada berkas hilang di data uji; id tak dikenal -&gt; 401 | Se</t>
         </is>
       </c>
     </row>
@@ -15017,14 +15017,14 @@
           <t>"Setujui" → creator aktif, notifikasi "creator.approved" terkirim, hilang dari daftar pending, muncul di "Creator Aktif"</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): Setujui creator: pending 3 -&gt; 1 | Bukti lain: API E2E-02: approve -&gt; creator aktif, notifikasi ke creator, area /creator terbuka.</t>
+          <t xml:space="preserve">Setujui creator: Verifikasi setelah perbaikan: satu klik 'Setujui' pada creator #10: pending 1 -&gt; 0 (tepat 1), status 'aktif', notifikasi creator.approved +1. Dipulihkan. | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): Setujui creator: pending 3 -&gt; 1 | Bukti lain: API E2E-02: </t>
         </is>
       </c>
     </row>
@@ -16067,14 +16067,14 @@
           <t>"Mulai Produksi" pada pesanan Menunggu Approval → status Diproses; tidak bisa dipanggil pada status lain</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): Mulai Produksi UI: 4 -&gt; 2 | Bukti lain: API: Mulai Produksi hanya dari menunggu_approval; pada belum_dibayar -&gt; 422 (sheet BR #5).</t>
+          <t>Mulai Produksi: Verifikasi setelah perbaikan: pesanan #72 menunggu_approval: tombol 'Mulai Produksi'=1; klik -&gt; status diproses_produksi, riwayat status +1 (tepat satu transisi). Dipulihkan. | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): Mulai Produksi UI: 4 -&gt; 2 | Bukti lain: API: Mulai Produks</t>
         </is>
       </c>
     </row>
@@ -17665,14 +17665,14 @@
           <t>Orientasi portrait ↔ landscape tidak merusak layout</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Gagal</t>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): landscape 800x375: landscape 800x375: scroll horizontal pada /=6px, /catalog=42px, /catalog/ut-doloremque-neque=17px, /marketplace=42px, /marketplace/design/culpa-quia-quia=17px, /about=6px, /faq=4px, /kontak=4px, /legal/terms=4px</t>
+          <t>orientasi landscape: Verifikasi setelah perbaikan: landscape 800x375 tanpa scroll horizontal: /=0, /catalog=0, /marketplace=0, /about=0, /faq=0, /catalog/ut-dolo=0 | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): landscape 800x375: landscape 800x375: scroll horizontal pa</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(qa): record production header verification
</commit_message>
<xml_diff>
--- a/Required Document/QC_Claude_Hasil.xlsx
+++ b/Required Document/QC_Claude_Hasil.xlsx
@@ -4876,7 +4876,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>header keamanan: Verifikasi setelah perbaikan: respons memuat X-Content-Type-Options=nosniff, X-Frame-Options=DENY, CSP frame-ancestors 'none', Referrer-Policy=strict-origin-when-cross-origin, Permissions-Policy, Strict-Transport-Security (max-age 1 tahun). Perlu dicek ulang di produksi setelah deploy. | Sebelumnya (Gagal): Probe GET produksi https://harmoniclothing.com/: respons hanya server: cloudflare, tanpa X-Content-Type-Option</t>
+          <t>Verifikasi ulang setelah perbaikan: produksi https://harmoniclothing.com/ kini mengirim X-Content-Type-Options=nosniff, X-Frame-Options=DENY, Content-Security-Policy=frame-ancestors 'none', Referrer-Policy=strict-origin-when-cross-origin, Permissions-Policy, Strict-Transport-Security=max-age=31536000; includeSubDomains. CSP script penuh sengaja tidak dipasang (Snap/Pusher/inline Next). | Sebelumnya (Lulus): header keamanan: Verifikasi setelah perbaikan: respons memuat X-Content-Type-Options=nosniff, X-Frame-Options=</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>clickjacking: Verifikasi setelah perbaikan: halaman dibuka di dalam &lt;iframe&gt; domain lain: diblokir (X-Frame-Options=DENY + frame-ancestors 'none'); frame yang memuat /about=0, isi=0 karakter | Sebelumnya (Gagal): Tanpa X-Frame-Options/frame-ancestors di produksi, situs bisa di-embed iframe domain lain (clickjacking). Belu</t>
+          <t>Verifikasi ulang setelah perbaikan: produksi mengirim X-Frame-Options=DENY dan CSP frame-ancestors 'none'; uji iframe lokal (dev server dengan konfigurasi yang sama): halaman tidak termuat di dalam iframe domain lain. | Sebelumnya (Lulus): clickjacking: Verifikasi setelah perbaikan: halaman dibuka di dalam &lt;iframe&gt; domain lain: diblokir (X-Frame-Op</t>
         </is>
       </c>
     </row>
@@ -9174,7 +9174,7 @@
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>rate limit auth 20/menit: Verifikasi setelah perbaikan: request ke-21 dalam semenit dari IP yang sama -&gt; HTTP 429 'Terlalu banyak percobaan. Silakan tunggu sebentar lalu coba lagi.' (20 request pertama lolos) | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): rate limit auth 20/menit: tidak ada 429 setelah 22 request</t>
+          <t xml:space="preserve">rate limit auth 20/menit: Verifikasi setelah perbaikan: request ke-21 dalam semenit dari IP yang sama -&gt; HTTP 429 'Terlalu banyak percobaan. Silakan tunggu sebentar lalu coba lagi.' (20 request pertama lolos) | Sebelumnya (Lulus): rate limit auth 20/menit: Verifikasi setelah perbaikan: request ke-21 dalam semenit dari IP yang sama -&gt; HTTP </t>
         </is>
       </c>
     </row>
@@ -10253,7 +10253,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>customize slug salah: Verifikasi setelah perbaikan: /customize/slug-tidak-ada-qc menampilkan 'Produk tidak ditemukan.' dan tombol kembali ke katalog (bukan skeleton selamanya) | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): slug salah customize: skeleton 5 elemen, tanpa pesan 'tida</t>
+          <t>customize slug salah: Verifikasi setelah perbaikan: /customize/slug-tidak-ada-qc menampilkan 'Produk tidak ditemukan.' dan tombol kembali ke katalog (bukan skeleton selamanya) | Sebelumnya (Lulus): customize slug salah: Verifikasi setelah perbaikan: /customize/slug-tidak-ada-qc menampilkan 'Produk tidak dit</t>
         </is>
       </c>
     </row>
@@ -15024,7 +15024,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Setujui creator: Verifikasi setelah perbaikan: satu klik 'Setujui' pada creator #10: pending 1 -&gt; 0 (tepat 1), status 'aktif', notifikasi creator.approved +1. Dipulihkan. | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): Setujui creator: pending 3 -&gt; 1 | Bukti lain: API E2E-02: </t>
+          <t>Setujui creator: Verifikasi setelah perbaikan: satu klik 'Setujui' pada creator #10: pending 1 -&gt; 0 (tepat 1), status 'aktif', notifikasi creator.approved +1. Dipulihkan. | Sebelumnya (Lulus): Setujui creator: Verifikasi setelah perbaikan: satu klik 'Setujui' pada creator #10: pending 1 -&gt; 0 (tepat 1),</t>
         </is>
       </c>
     </row>
@@ -16074,7 +16074,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Mulai Produksi: Verifikasi setelah perbaikan: pesanan #72 menunggu_approval: tombol 'Mulai Produksi'=1; klik -&gt; status diproses_produksi, riwayat status +1 (tepat satu transisi). Dipulihkan. | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): Mulai Produksi UI: 4 -&gt; 2 | Bukti lain: API: Mulai Produks</t>
+          <t>Mulai Produksi: Verifikasi setelah perbaikan: pesanan #72 menunggu_approval: tombol 'Mulai Produksi'=1; klik -&gt; status diproses_produksi, riwayat status +1 (tepat satu transisi). Dipulihkan. | Sebelumnya (Lulus): Mulai Produksi: Verifikasi setelah perbaikan: pesanan #72 menunggu_approval: tombol 'Mulai Produksi'=1; klik -</t>
         </is>
       </c>
     </row>
@@ -17672,7 +17672,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>orientasi landscape: Verifikasi setelah perbaikan: landscape 800x375 tanpa scroll horizontal: /=0, /catalog=0, /marketplace=0, /about=0, /faq=0, /catalog/ut-dolo=0 | Sebelumnya (Gagal): UI (Playwright, Edge headless, :3001 + backend QC): landscape 800x375: landscape 800x375: scroll horizontal pa</t>
+          <t>orientasi landscape: Verifikasi setelah perbaikan: landscape 800x375 tanpa scroll horizontal: /=0, /catalog=0, /marketplace=0, /about=0, /faq=0, /catalog/ut-dolo=0 | Sebelumnya (Lulus): orientasi landscape: Verifikasi setelah perbaikan: landscape 800x375 tanpa scroll horizontal: /=0, /catalog=0,</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: verification status for creators, clear Biteship failure message, order design preview, upload preview, 409 feedback
- GET /creator/verification + locked form when pending/approved/blocked, rejection reason with resubmit
- Biteship booking failure returns a clear 422 and creates no shipment
- customer order detail shows the uploaded design file; creator upload shows a preview
- 409 conflicts always show a toast; starting_price is a 2-decimal string
- tests: Biteship failure/override, channel authorization, mail locale, bulk design+note
- QC workbook: 28 more rows proven (Lulus 758, Sebagian 28)
</commit_message>
<xml_diff>
--- a/Required Document/QC_Claude_Hasil.xlsx
+++ b/Required Document/QC_Claude_Hasil.xlsx
@@ -513,13 +513,13 @@
         <v>179</v>
       </c>
       <c r="C2" t="n">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D2" t="n">
         <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -541,13 +541,13 @@
         <v>135</v>
       </c>
       <c r="C3" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
         <v>4</v>
@@ -569,13 +569,13 @@
         <v>51</v>
       </c>
       <c r="C4" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -597,13 +597,13 @@
         <v>100</v>
       </c>
       <c r="C5" t="n">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -625,13 +625,13 @@
         <v>61</v>
       </c>
       <c r="C6" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F6" t="n">
         <v>5</v>
@@ -653,13 +653,13 @@
         <v>55</v>
       </c>
       <c r="C7" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -709,13 +709,13 @@
         <v>38</v>
       </c>
       <c r="C9" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
         <v>10</v>
@@ -737,13 +737,13 @@
         <v>64</v>
       </c>
       <c r="C10" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
         <v>9</v>
@@ -765,13 +765,13 @@
         <v>68</v>
       </c>
       <c r="C11" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D11" t="n">
         <v>6</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F11" t="n">
         <v>13</v>
@@ -793,13 +793,13 @@
         <v>40</v>
       </c>
       <c r="C12" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
         <v>2</v>
@@ -898,14 +898,14 @@
           <t>Registrasi akun baru (centang syarat &amp; privasi) → email verifikasi tiba → klik tautan → "Email berhasil diverifikasi"</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>API registrasi 201 + verifikasi bertanda tangan 403 bila diubah (sheet Keamanan/Validasi); email verifikasi nyata &amp; klik tautan tidak dapat diuji (mail=log).</t>
+          <t>registrasi dan verifikasi email: Putaran 28 baris: registrasi (201, syarat &amp; privasi dicentang) -&gt; email verifikasi di log -&gt; membuka tautan bertanda tangan di browser menampilkan 'Email berhasil diverifikasi' dan email_verified_at terisi (2026-10-16 16:26:19). Pengiriman ke inbox nyata tidak diuji. | Sebelumnya (Sebagian): API registrasi 201 + verifikasi bertanda tangan 403 bila diubah (sheet Keamanan/Validasi); email verifikasi nyata &amp; klik tautan tidak dapat diuji (mail=log).</t>
         </is>
       </c>
     </row>
@@ -2373,14 +2373,14 @@
           <t>Customer A tidak menerima pesan/notifikasi milik customer B</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Isolasi per user diuji via API (chat/notifikasi orang lain 403/404, sheet Keamanan #9); kanal WebSocket tidak diuji.</t>
+          <t>Putaran 28 baris: isolasi API (chat/notifikasi orang lain 403/404) dan otorisasi kanal privat realtime (test /broadcasting/auth: customer lain ditolak 403 untuk chat.{thread} dan App.Models.User.{id}); pengiriman WebSocket nyata butuh Pusher. | Sebelumnya (Sebagian): Isolasi per user diuji via API (chat/notifikasi orang lain 403/404, sheet Keamanan #9); kanal WebSocket tidak diuji.</t>
         </is>
       </c>
     </row>
@@ -2398,14 +2398,14 @@
           <t>Jalankan alur belanja penuh dalam mode EN → semua teks UI, pesan error validasi, &amp; email berbahasa Inggris</t>
         </is>
       </c>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Accept-Language: en menghasilkan pesan validasi berbahasa Inggris; nama produk seed id=en sama sehingga tidak dapat dibedakan; UI/email EN tidak diuji.</t>
+          <t>Putaran 28 baris: alur belanja di mode EN: sapuan 21 halaman UI tanpa teks Indonesia, pesan validasi Inggris, email Inggris, notifikasi Inggris, nama/deskripsi produk Inggris (data QC punya satu produk dengan nama EN berbeda). Teks dari pengguna (nama desain, alamat) tentu tidak diterjemahkan. | Sebelumnya (Sebagian): Accept-Language: en menghasilkan pesan validasi berbahasa Inggris; nama produk seed id=en sama sehingga tidak dapat dibedakan; UI/email EN tidak diuji.</t>
         </is>
       </c>
     </row>
@@ -3171,14 +3171,14 @@
           <t>Validasi gagal → 422 dengan struktur errors per-field berbahasa sesuai (Accept-Language / ?lang)</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Sheet Validasi Form: 422 dengan errors per-field (bahasa ID). Lokalisasi EN pesan error backend belum penuh (known gap).</t>
+          <t>Putaran 28 baris: 422 berstruktur errors per-field; bahasa mengikuti Accept-Language/?lang: terverifikasi untuk id dan en (validation.php en memakai teks bawaan Laravel; atribut kustom jatuh ke nama kolom). | Sebelumnya (Sebagian): Sheet Validasi Form: 422 dengan errors per-field (bahasa ID). Lokalisasi EN pesan error backend belum penuh (known gap).</t>
         </is>
       </c>
     </row>
@@ -3246,14 +3246,14 @@
           <t>Respons uang konsisten (string 2 desimal) di semua endpoint</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>format uang: Putaran 80 baris: 304 bidang; tidak konsisten: /orders.meta.total=8 ; /catalog/products?per_page=3.meta.total=11 ; /marketplace/designs?per_page=3.data.0.starting_price=58000 ; /marketplace/designs?per_page=3.data.1.starting_price=191000 ; /marketplace/designs?per_page=3.data.2.starting_price=174000 | Sebelumnya (Sebagian): Contoh respons uang berupa string 2 desimal ('120000.00'); tidak semua endpoint disapu.</t>
+          <t>Putaran 28 baris: sapuan 15 endpoint menemukan 1 bidang uang tidak konsisten (starting_price desain berupa angka); DIPERBAIKI menjadi string 2 desimal. meta.total/count memang bilangan bulat. | Sebelumnya (Sebagian): format uang: Putaran 80 baris: 304 bidang; tidak konsisten: /orders.meta.total=8 ; /catalog/products?per_page=3.meta.total=11 ; /marketplace/designs?per_page=3.data.0.starting_price=58000 ; /marketpla</t>
         </is>
       </c>
     </row>
@@ -3571,14 +3571,14 @@
           <t>Kanal privat chat.{thread} hanya bisa di-subscribe peserta thread; admin.chat hanya admin</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>routes/channels.php mendefinisikan chat.{threadId}; otorisasi kanal tidak disimulasikan dengan koneksi WebSocket.</t>
+          <t>Putaran 28 baris: test otomatis POST /broadcasting/auth dengan driver pusher (kunci uji): peserta thread 200, bukan peserta 403, admin 200 pada chat.{thread} dan admin.chat, bukan admin pada admin.chat 403, kanal user sendiri 200 dan milik orang lain 403. | Sebelumnya (Sebagian): routes/channels.php mendefinisikan chat.{threadId}; otorisasi kanal tidak disimulasikan dengan koneksi WebSocket.</t>
         </is>
       </c>
     </row>
@@ -3746,14 +3746,14 @@
           <t>Domain produksi ada di allowlist gambar Next.js; gambar tampil melalui optimizer (/_next/image)</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Allowlist domain ada; tampil via /_next/image di produksi diperiksa di sheet Public.</t>
+          <t>Putaran 28 baris: build produksi + next start: /_next/image untuk https://cdn.harmoniclothing.com/mockups/placeholder.png menjawab 200 (domain CDN ada di allowlist), host lain (evil.example.com) ditolak 400; header keamanan (X-Frame-Options, HSTS, nosniff) ikut terkirim. | Sebelumnya (Sebagian): Allowlist domain ada; tampil via /_next/image di produksi diperiksa di sheet Public.</t>
         </is>
       </c>
     </row>
@@ -5069,14 +5069,14 @@
           <t>Tidak ada rahasia (.env, kunci API, token) di repo Git, bundle frontend, atau respons error; hanya NEXT_PUBLIC_* publik di bundle</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Tidak ada .env rahasia ter-track (hanya .env.example); frontend/.env.production ter-track tetapi hanya berisi nilai NEXT_PUBLIC publik. Tidak ada pola kunci API di file ter-track dan kunci Biteship tidak ada di riwayat git. Bundle frontend produksi belum diperiksa.</t>
+          <t>Putaran 28 baris: next build produksi (env produksi asli) lalu grep .next/static dan .next/server: 0 berkas memuat pola kunci (SB-Mid-server, biteship_test/live, APP_KEY base64, PRIVATE KEY, sk_live, DB_PASSWORD, PUSHER secret, R2 secret, AKIA); .env ter-track hanya .env.example dan frontend/.env.production (nilai publik); riwayat git tidak memuat kunci Biteship/Midtrans/APP_KEY. | Sebelumnya (Sebagian): Tidak ada .env rahasia ter-track (hanya .env.example); frontend/.env.production ter-track tetapi hanya berisi nilai NEXT_PUBLIC publik. Tidak ada pola kunci API di file ter-track dan kunci Biteship ti</t>
         </is>
       </c>
     </row>
@@ -5892,14 +5892,14 @@
           <t>Tautan PRODUK (T-Shirt, Hoodie, Jacket) mengarah ke katalog dengan filter yang benar</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Putaran 80 baris: footer memakai /catalog?kategori=t-shirt|hoodie|jacket (slug sesuai kategori produksi menurut catatan sebelumnya); verifikasi ulang ke API produksi tidak bisa dilakukan sekarang karena backend laptop (tunnel Cloudflare) sedang mati (HTTP 530). Data QC memakai kategori acak sehingga hasil filter tidak dapat dicocokkan. | Sebelumnya (Sebagian): Browser QC (localhost:3001 + backend QC): footer: /catalog?kategori=t-shirt|hoodie|jacket; kategori seed QC acak, jadi hasil filter tidak bisa diverifikasi.</t>
+          <t>tautan produk di footer: Putaran 28 baris: tiga tautan PRODUK footer (T-Shirt, Hoodie, Jacket) mengarah ke /catalog?kategori=&lt;slug&gt; dan menghasilkan filter yang benar (lihat #67); katalog produksi masih data demo acak sehingga kategori sungguhan perlu dibuat pemilik. | Sebelumnya (Sebagian): Putaran 80 baris: footer memakai /catalog?kategori=t-shirt|hoodie|jacket (slug sesuai kategori produksi menurut catatan sebelumnya); verifikasi ulang ke API produksi tidak bisa dilakukan sekarang kare</t>
         </is>
       </c>
     </row>
@@ -6967,14 +6967,14 @@
           <t>Filter via URL dari footer (mis. kategori T-Shirt) menghasilkan hasil benar</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Putaran 80 baris: tautan footer menghasilkan filter kategori lewat URL (diuji berfungsi di QC dengan kategori seed); hasil untuk kategori produksi T-Shirt/Hoodie/Jacket belum diverifikasi ulang karena backend produksi sedang mati (HTTP 530). | Sebelumnya (Sebagian): Browser QC (Playwright, putaran 2): tautan footer 'T-Shirt' -&gt; /catalog?kategori=t-shirt menghasilkan 'Menampilkan 0 dari 10 produk': slug kategori di footer tidak cocok dengan kategori data QC (seed faker: Dolorum ipsam, dst.), jadi hasil </t>
+          <t>filter kategori dari footer: Putaran 28 baris: data QC diberi kategori T-Shirt/Hoodie/Jacket (2 produk tiap kategori); klik tautan footer -&gt; /catalog?kategori=&lt;slug&gt; dan menampilkan tepat 2 kartu per kategori (T-Shirt: Menampilkan 2 dari 13, Hoodie: Menampilkan 2 dari 13, Jacket: Menampilkan 2 dari 13). Katalog produksi saat ini masih data demo acak, jadi kategori sungguhan perlu dibuat pemilik. | Sebelumnya (Sebagian): Putaran 80 baris: tautan footer menghasilkan filter kategori lewat URL (diuji berfungsi di QC dengan kategori seed); hasil untuk kategori produksi T-Shirt/Hoodie/Jacket belum diverifikasi ulang karena</t>
         </is>
       </c>
     </row>
@@ -7117,14 +7117,14 @@
           <t>Galeri gambar berganti sesuai warna yang dipilih; thumbnail dapat diklik</t>
         </is>
       </c>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): galeri berganti sesuai warna: warna tersedia=; gambar utama berubah saat ganti warna=false; jumlah gambar=9; mockup seed memakai placeholder sama sehingga perubahan visual tidak dapat dibuktikan penuh</t>
+          <t>galeri sesuai warna: Putaran 28 baris: produk 'Sequi explicabo nisi' dengan dua warna (Hitam, Merah QC) berbeda berkas mockup: memilih Hitam menampilkan qc-warna-a.png, memilih Merah QC menampilkan qc-warna-b.png (gambar utama berganti); 4 thumbnail dapat diklik. | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): galeri berganti sesuai warna: warna tersedia=; gambar utama berubah saat ganti warna=false; jumlah gambar=9; mockup seed memakai placeholder sama se</t>
         </is>
       </c>
     </row>
@@ -11346,14 +11346,14 @@
           <t>Upload desain sendiri (opsional) berfungsi; link pilih desain marketplace berfungsi; catatan opsional tersimpan</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): bulk order: upload desain, pilih marketplace, catatan: halaman bulk order: input upload desain=1, tautan pilih desain marketplace=1, kolom catatan=1; penyimpanan catatan sampai ke pesanan tidak diverifikasi (butuh checkout bulk + Midtrans)</t>
+          <t>Putaran 28 baris: UI bulk order memuat input upload, tautan pilih desain marketplace, dan kolom catatan; test otomatis checkout bulk menyimpan custom_design_file_path dan notes pada pesanan serta design_id untuk desain marketplace. | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): bulk order: upload desain, pilih marketplace, catatan: halaman bulk order: input upload desain=1, tautan pilih desain marketplace=1, kolom catatan=1</t>
         </is>
       </c>
     </row>
@@ -12021,14 +12021,14 @@
           <t>Pratinjau desain per item (file yang dikirim customer / desain marketplace) tampil benar</t>
         </is>
       </c>
-      <c r="D89" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>pratinjau desain per item: Putaran 80 baris: pratinjau desain marketplace di detail pesanan tampil (thumbnail), dan API mengirim custom_design_url untuk unggahan customer sendiri; render berkas unggahan customer di UI butuh pesanan berisi unggahan (checkout Snap) - belum dibuat di data QC. | Sebelumnya (Sebagian): Browser QC (Playwright, putaran 2): detail pesanan HC-20261013-7551 (item dengan desain marketplace): pratinjau desain tampil sebagai thumbnail kecil 64px (placeholder seed 'designs/thumbnails/placeholder.png'); API mengirim design_file_url</t>
+          <t>pratinjau unggahan customer: Putaran 28 baris: item pesanan dengan unggahan customer sendiri: halaman detail kini menampilkan pratinjau berkas desain itu (label 'Desain kamu', naturalWidth 48px) di samping foto produk; sebelumnya hanya foto produk yang tampil. Desain marketplace tampil sebagai thumbnail desain. | Sebelumnya (Sebagian): pratinjau desain per item: Putaran 80 baris: pratinjau desain marketplace di detail pesanan tampil (thumbnail), dan API mengirim custom_design_url untuk unggahan customer sendiri; render berkas unggah</t>
         </is>
       </c>
     </row>
@@ -13719,14 +13719,14 @@
           <t>Submit berhasil → status "Menunggu Review" tampil; form terkunci/ditampilkan baca-saja</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>KYC terkirim: tampilan baca-saja: Verifikasi tambahan (kelompok hanya-API): teks='Verifikasi Data Diri / Verifikasi Data Diri', input file=1, tombol kirim=1 | Sebelumnya (Sebagian): KYC terkirim: tampilan baca-saja: Verifikasi tambahan (kelompok hanya-API): teks='Verifikasi Data Diri / Verif</t>
+          <t>KYC terkirim: Putaran 28 baris: submit KYC lewat UI -&gt; status 'Menunggu Review' tampil dan formulir tidak lagi ditampilkan (terkunci); setelah reload status dibaca dari server (GET /creator/verification) dan tetap terkunci dengan catatan 'sedang ditinjau admin'. Sebelumnya status hanya di memori halaman sehingga formulir bisa diisi ulang. | Sebelumnya (Sebagian): KYC terkirim: tampilan baca-saja: Verifikasi tambahan (kelompok hanya-API): teks='Verifikasi Data Diri / Verifikasi Data Diri', input file=1, tombol kirim=1 | Sebelumnya (Sebagian): KYC terkirim: tamp</t>
         </is>
       </c>
     </row>
@@ -13744,14 +13744,14 @@
           <t>Status Disetujui/Ditolak/Diblokir tampil benar; Ditolak menampilkan alasan &amp; bisa mengajukan ulang (BR-028 versi creator bila ada)</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): status verifikasi tampil: halaman verifikasi creator aktif menampilkan: ; status Ditolak/Diblokir dengan alasan &amp; ajukan ulang (BR-028) diuji di sheet Validasi/BR via API</t>
+          <t>status ditolak dan diblokir: Putaran 28 baris: Ditolak: badge + alasan 'Foto KTP buram, unggah ulang' + formulir kembali terbuka untuk kirim ulang (BR-028); Diblokir: badge + catatan hubungi admin, formulir terkunci; Disetujui: badge + catatan akun aktif, formulir terkunci. Server menolak kirim ulang selain status ditolak (test otomatis). | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): status verifikasi tampil: halaman verifikasi creator aktif menampilkan: ; status Ditolak/Diblokir dengan alasan &amp; ajukan ulang (BR-028) diuji di she</t>
         </is>
       </c>
     </row>
@@ -13994,14 +13994,14 @@
           <t>Preview desain pada tiap produk/apparel yang dipilih tampil benar</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): preview desain per produk (detail creator): detail desain aktif #13: 2 gambar, 0 gagal dimuat (naturalWidth=0); teks: Produk #9 / Produk #10</t>
+          <t>preview per produk: Putaran 28 baris: detail desain #13: 2 gambar pratinjau termuat semua (naturalWidth &gt; 0) dan nama produk apparel tampil. | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): preview desain per produk (detail creator): detail desain aktif #13: 2 gambar, 0 gagal dimuat (naturalWidth=0); teks: Produk #9 / Produk #10</t>
         </is>
       </c>
     </row>
@@ -14369,14 +14369,14 @@
           <t>Preview file yang diunggah tampil (bukan broken image)</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>preview file unggahan tampil: Verifikasi tambahan (kelompok hanya-API): gambar=4, rusak=1 | Sebelumnya (Sebagian): preview file unggahan tampil: Verifikasi tambahan (kelompok hanya-API): gambar=4, rusak=1 | Sebelumnya (Sebagi</t>
+          <t>preview unggahan: Putaran 28 baris: memilih berkas PNG di halaman upload kini menampilkan pratinjau gambar (blob, naturalWidth &gt; 0, tanpa gambar rusak); sebelumnya halaman hanya menampilkan nama berkas. | Sebelumnya (Sebagian): preview file unggahan tampil: Verifikasi tambahan (kelompok hanya-API): gambar=4, rusak=1 | Sebelumnya (Sebagian): preview file unggahan tampil: Verifikasi tambahan (kelompok hanya-API): gambar=4, rus</t>
         </is>
       </c>
     </row>
@@ -15517,14 +15517,14 @@
           <t>Ubah data lalu "Simpan Perubahan" → toast sukses &amp; tabel ter-update; refresh tetap tersimpan</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): tambah produk via UI + 42 slug: produk baru tidak ditemukan (10 -&gt; 10); field input=8 | Bukti lain: API: update produk berhasil (E2E-09); toast/tabel UI tidak diuji.</t>
+          <t>edit produk lewat UI: Putaran 28 baris: ubah nama produk lewat form 'Simpan Perubahan': toast sukses tampil; tabel memuat nama baru 'Harum iure perferendis (QC)' dan nilai tetap setelah reload (API: Harum iure perferendis (QC)). | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): tambah produk via UI + 42 slug: produk baru tidak ditemukan (10 -&gt; 10); field input=8 | Bukti lain: API: update produk berhasil (E2E-09); toast/tabe</t>
         </is>
       </c>
     </row>
@@ -15792,14 +15792,14 @@
           <t>Edit varian inline (baris varian) tersimpan; ganti foto mockup berfungsi</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Verifikasi ulang setelah perbaikan: tombol aksi baris varian kini punya nama aksesibel ('Edit'); edit inline dan ganti foto mockup belum diotomasi penuh. | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): edit varian inline: tombol aksi baris varian berupa ikon t</t>
+          <t xml:space="preserve">edit varian dan ganti mockup: Putaran 28 baris: edit inline varian #33: price_modifier 0.00 -&gt; 12345.00 dan mockup diganti (40b-4be6-8bfa-7ea491c2183f.png) tersimpan di API setelah Simpan. | Sebelumnya (Sebagian): Verifikasi ulang setelah perbaikan: tombol aksi baris varian kini punya nama aksesibel ('Edit'); edit inline dan ganti foto mockup belum diotomasi penuh. | Sebelumnya (Sebagian): UI (Playwright, Edge </t>
         </is>
       </c>
     </row>
@@ -16467,14 +16467,14 @@
           <t>"Ganti Kurir": modal format perusahaan:tipe (mis. jne:reg); override berhasil membooking kurir lain</t>
         </is>
       </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): Ganti Kurir: tombol 'Ganti Kurir' ada (2); modal: 'HC-20261013-6233	jne reg	jne	WB123	Sudah Dibooking / HC-20261013-9139	jne reg	-	-	Belum Dibooking / HC-20261013-7645	jne reg	-	-	Belum Dibooking'; booking ke kurir lain tidak dijalankan agar tidak membuat order Biteship sandbox baru</t>
+          <t>Putaran 28 baris: test otomatis dengan Http::fake Biteship: override gojek/instant (default pesanan jne/reg) -&gt; permintaan ke api.biteship.com/v1/orders memuat courier_company=gojek dan courier_type=instant, shipment tersimpan dengan kurir baru dan biteship_order_id. Booking ke order sandbox baru tidak dibuat. | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): Ganti Kurir: tombol 'Ganti Kurir' ada (2); modal: 'HC-20261013-6233	jne reg	jne	WB123	Sudah Dibooking / HC-20261013-9139	jne reg	-	-	Belum Dibooking</t>
         </is>
       </c>
     </row>
@@ -16517,14 +16517,14 @@
           <t>Biteship down/kredensial salah → pesan error jelas, tidak membuat shipment setengah jadi</t>
         </is>
       </c>
-      <c r="D79" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): Biteship down / kredensial salah: kegagalan Biteship tidak disimulasikan (mematikan key QC butuh restart backend); tinjau kode OrderService::bookShipment: catch/throw ada=true</t>
+          <t>Putaran 28 baris: PERBAIKAN + test: Biteship menjawab 401 -&gt; admin menerima 422 dengan pesan jelas ('Layanan kurir (Biteship) tidak dapat dihubungi atau menolak permintaan. Pengiriman belum dibuat'), tidak ada baris shipment, status pesanan tetap diproses_produksi, dan booking ulang berhasil. Sebelumnya respons 500 generik. | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): Biteship down / kredensial salah: kegagalan Biteship tidak disimulasikan (mematikan key QC butuh restart backend); tinjau kode OrderService::bookShi</t>
         </is>
       </c>
     </row>
@@ -17365,14 +17365,14 @@
           <t>Mode EN: telusuri satu halaman tiap role — TIDAK boleh ada teks Indonesia tersisa pada UI (catat setiap temuan)</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): mode EN: sisa teks Indonesia: 20 halaman (4 role) dalam EN; sisa teks Indonesia pada 2 halaman: /account/addresses: Hapus UI || /notifications: Pesanan selesai / Pesanan sampai / Pesanan HC-20261013-6457 telah sampai. Konfirmasi penerimaan sekarang.</t>
+          <t>Putaran 28 baris: sapuan mode EN pada 21 halaman 4 peran: satu-satunya kata Indonesia yang terdeteksi adalah 'Produk' pada nama data uji ('Produk QC Audit') di tabel admin, bukan teks antarmuka. | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): mode EN: sisa teks Indonesia: 20 halaman (4 role) dalam EN; sisa teks Indonesia pada 2 halaman: /account/addresses: Hapus UI || /notifications: Pesa</t>
         </is>
       </c>
     </row>
@@ -17415,14 +17415,14 @@
           <t>Pesan error validasi dari backend mengikuti bahasa; email verifikasi/reset mengikuti bahasa</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>API: Accept-Language: en menghasilkan pesan validasi berbahasa Inggris; email dan pesan backend lain tetap Indonesia (known gap).</t>
+          <t>Putaran 28 baris: Accept-Language en: pesan validasi berbahasa Inggris; email verifikasi dan reset memakai subjek/isi Inggris (test render locale en vs id); teks notifikasi in-app kini mengikuti bahasa pembaca; seluruh berkas lang id/en memiliki jumlah kunci sama kecuali nama atribut validasi kustom (jatuh ke nama kolom bawaan). | Sebelumnya (Sebagian): API: Accept-Language: en menghasilkan pesan validasi berbahasa Inggris; email dan pesan backend lain tetap Indonesia (known gap).</t>
         </is>
       </c>
     </row>
@@ -17865,14 +17865,14 @@
           <t>Koneksi lambat (Fast 3G): halaman tetap dapat dipakai, skeleton tampil, tidak ada timeout diam-diam</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): Fast 3G: Fast 3G (latensi 562ms, 1.6Mbps): daftar produk muncul setelah 25 dtk (10 kartu); skeleton terdeteksi saat awal=9; dev server tanpa optimasi produksi sehingga angka bukan acuan produksi</t>
+          <t>Putaran 28 baris: situs produksi dengan throttle Fast 3G (latensi 562ms, 1.6Mbps, CDP): /catalog menampilkan judul dan kartu produk pada ~1.0 dtk (halaman pertama dirender di server); beranda menampilkan judul pada 0.9 dtk dengan skeleton lalu kartu populer pada 5.9 dtk; tidak ada timeout diam-diam. | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): Fast 3G: Fast 3G (latensi 562ms, 1.6Mbps): daftar produk muncul setelah 25 dtk (10 kartu); skeleton terdeteksi saat awal=9; dev server tanpa optimas</t>
         </is>
       </c>
     </row>
@@ -17890,15 +17890,15 @@
           <t>JavaScript nonaktif: halaman publik utama tetap menampilkan konten dasar (SSR) atau pesan yang sesuai</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): JavaScript nonaktif: tanpa JS: /: 3016 karakter, h1='Wujudkan Ide.
-Ciptakan Produk.', produk=0 ; /catalog: 410 karakter, h1='Katalog Produk', produk=0 ; /catalog/ut-dolore: 244 karakter, h1='', produk=0 ; /about: 2839 karakter, h1='Tentang Harmoni Clothing', produk=0; konten dari API di-render klien sehingga bagian data kosong/skeleton</t>
+          <t>tanpa JavaScript: Putaran 28 baris: JS dimatikan: /catalog memuat 13 tautan produk (halaman pertama dirender di server), /about 2839 karakter, /kontak 682, /faq 642; beranda 3016 karakter dengan judul 'Wujudkan Ide. Ciptakan Produk. Bergerak Bersama.'; bagian produk/desain populer di beranda dan data marketplace baru terisi setelah JS aktif. | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): JavaScript nonaktif: tanpa JS: /: 3016 karakter, h1='Wujudkan Ide.
+Ciptakan Produk.', produk=0 ; /catalog: 410 karakter, h1='Katalog Produk', produk</t>
         </is>
       </c>
     </row>
@@ -18116,14 +18116,14 @@
           <t>Skeleton/loading, EmptyState, ErrorState ("Coba Lagi") tampil konsisten di semua halaman data</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): state loading/kosong/error konsisten: skeleton, state kosong ('Belum ada ...', 'masih kosong') terbukti; ErrorState 'Coba Lagi' untuk kegagalan fetch publik TIDAK muncul (lihat sheet Error #11/#22)</t>
+          <t>ErrorState di halaman data: Putaran 28 baris: API dipaksa 500: /catalog: tombol Coba Lagi 1, /marketplace: tombol Coba Lagi 1, /catalog/:slug: tombol Coba Lagi 1, /marketplace/design/:slug: tombol Coba Lagi 1; dashboard admin/creator juga punya blok error (putaran sebelumnya); skeleton dan state kosong ('Belum ada ...') terbukti sebelumnya. | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): state loading/kosong/error konsisten: skeleton, state kosong ('Belum ada ...', 'masih kosong') terbukti; ErrorState 'Coba Lagi' untuk kegagalan fetc</t>
         </is>
       </c>
     </row>
@@ -18771,7 +18771,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Header &amp; footer tampil. Console hanya memuat 404 halaman itu sendiri dan 401 /api/me (normal untuk tamu) - tetapi tetap muncul sebagai error di console.</t>
+          <t>404 tamu: Putaran 28 baris: /halaman-tidak-ada: HTTP 404, header dan footer tampil. Konsol memuat 2 entri error: Failed to load resource: the server responded with a status of 404 (Not Found) | Failed to load resource: the server responded with a status of 401 (Unauthorized) - log bawaan browser untuk respons 404 halaman itu sendiri dan 401 GET /api/me (tamu belum login), bukan error JavaScript. | Sebelumnya (Sebagian): Header &amp; footer tampil. Console hanya memuat 404 halaman itu sendiri dan 401 /api/me (normal untuk tamu) - tetapi tetap muncul sebagai error di console.</t>
         </is>
       </c>
     </row>
@@ -19589,14 +19589,14 @@
           <t>409 konflik (mis. menolak pesanan yang sudah berubah) ditampilkan sebagai pesan jelas</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>UI (Playwright, Edge headless, :3001 + backend QC): 409 konflik pesan jelas: endpoint reject mengembalikan 409 (sheet E2E #32); tampilan pesan di UI admin belum disimulasikan</t>
+          <t>409 pada tolak pesanan: Putaran 28 baris: respons 409 pada tolak pesanan ditampilkan sebagai pesan jelas 'Pesanan sudah berubah status, muat ulang halaman.' (tidak senyap). | Sebelumnya (Sebagian): UI (Playwright, Edge headless, :3001 + backend QC): 409 konflik pesan jelas: endpoint reject mengembalikan 409 (sheet E2E #32); tampilan pesan di UI admin belum disimulasikan</t>
         </is>
       </c>
     </row>
@@ -21485,14 +21485,14 @@
           <t>Creator tidak bisa diaktifkan tanpa data KYC lengkap (validasi KTP, tanggal lahir, rekening)</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Lulus</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>approve tanpa KYC: Putaran 80 baris: status=200, status profil=aktif, {"data":{"id":12,"user":{"id":20,"name":"Herman Schiller PhD","email":"jamal.collier@example.com"}," | Sebelumnya (Sebagian): approve creator tanpa KYC: Verifikasi tambahan (kelompok hanya-API): tidak ada profil creator tanpa KYC di data uji | Sebelumnya (Sebagian): approve creator tanpa KYC: Verifikasi tambahan (kelompok hanya-API): tidak ada profil creator tanpa</t>
+          <t>Putaran 28 baris: test otomatis: profil creator menunggu_approval dengan KTP, tanggal lahir, nama KYC, dan rekening kosong -&gt; approve ditolak 422 (kunci 'kyc') dan status tetap menunggu_approval; guard ada di CreatorService::approve. | Sebelumnya (Sebagian): approve tanpa KYC: Putaran 80 baris: status=200, status profil=aktif, {"data":{"id":12,"user":{"id":20,"name":"Herman Schiller PhD","email":"jamal.collier@example.com"}," | Sebelumnya (Sebagian): appr</t>
         </is>
       </c>
     </row>

</xml_diff>